<commit_message>
Picks data, 2026-10-21 22:51 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$116</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -151,6 +151,24 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -728,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -762,7 +780,7 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>Today's rule: No rule yet (no graded picks).</t>
+          <t>Today's rule: Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
         </is>
       </c>
     </row>
@@ -790,19 +808,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H116)</f>
+        <f>SUM(H9:H118)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I116,"W")/(COUNTIF(I9:I116,"W")+COUNTIF(I9:I116,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I118,"W")/(COUNTIF(I9:I118,"W")+COUNTIF(I9:I118,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I116,"W")&amp;"-"&amp;COUNTIF(I9:I116,"L")</f>
+        <f>COUNTIF(I9:I118,"W")&amp;"-"&amp;COUNTIF(I9:I118,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I116,"W")+COUNTIF(I9:I116,"L")</f>
+        <f>COUNTIF(I9:I118,"W")+COUNTIF(I9:I118,"L")</f>
         <v/>
       </c>
     </row>
@@ -6052,8 +6070,104 @@
       </c>
       <c r="L116" s="13" t="inlineStr"/>
     </row>
+    <row r="117">
+      <c r="A117" s="10" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>PHI @ BUF</t>
+        </is>
+      </c>
+      <c r="C117" s="12" t="n">
+        <v>69.78</v>
+      </c>
+      <c r="D117" s="12" t="n">
+        <v>62.46</v>
+      </c>
+      <c r="E117" s="12">
+        <f>IF(OR(C117="",D117=""),"",ABS(C117-D117))</f>
+        <v/>
+      </c>
+      <c r="F117" s="13" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="G117" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="H117" s="15">
+        <f>IF(OR(F117="",G117="",AND(I117&lt;&gt;"W",I117&lt;&gt;"L")),"",IF(I117="W",IF(G117&gt;0,G117/100,1),IF(G117&lt;0,G117/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I117" s="13" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J117" s="11" t="inlineStr">
+        <is>
+          <t>PHI 3, BUF 1</t>
+        </is>
+      </c>
+      <c r="K117" s="11" t="inlineStr">
+        <is>
+          <t>DraftKings closing (missed the pick-time run)</t>
+        </is>
+      </c>
+      <c r="L117" s="13" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="10" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B118" s="11" t="inlineStr">
+        <is>
+          <t>FLA @ OTT</t>
+        </is>
+      </c>
+      <c r="C118" s="12" t="n">
+        <v>99.62</v>
+      </c>
+      <c r="D118" s="12" t="n">
+        <v>69.39</v>
+      </c>
+      <c r="E118" s="12">
+        <f>IF(OR(C118="",D118=""),"",ABS(C118-D118))</f>
+        <v/>
+      </c>
+      <c r="F118" s="13" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="G118" s="14" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H118" s="15">
+        <f>IF(OR(F118="",G118="",AND(I118&lt;&gt;"W",I118&lt;&gt;"L")),"",IF(I118="W",IF(G118&gt;0,G118/100,1),IF(G118&lt;0,G118/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I118" s="13" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J118" s="11" t="inlineStr">
+        <is>
+          <t>FLA 1, OTT 5</t>
+        </is>
+      </c>
+      <c r="K118" s="11" t="inlineStr">
+        <is>
+          <t>DraftKings closing (missed the pick-time run)</t>
+        </is>
+      </c>
+      <c r="L118" s="13" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L116"/>
+  <autoFilter ref="A8:L118"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -6062,7 +6176,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H116">
+  <conditionalFormatting sqref="H9:H118">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -6080,7 +6194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6134,6 +6248,38 @@
         <is>
           <t>Their units</t>
         </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>46-18, +23.02 units</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>66-42, +11.47 units</t>
+        </is>
+      </c>
+      <c r="E4" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A4)</f>
+        <v/>
+      </c>
+      <c r="F4" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A4,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A4,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G4" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A4)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -65712,105 +65858,105 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>How it works</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="17" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>System</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>In every game, pick the team whose team score was higher in its own previous game that season.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>Team score</t>
         </is>
       </c>
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>The website's formula and constants (dashboard_template.html, teamScore): 70 + 2.896 x goal difference (no empty-net goals, no shootout) + 1.997 x expected goals difference + 0.294 x score-adjusted 5-on-5 shot attempt difference, kept between 0 and 100. The constants were fitted on every game of 2025-26 (all 32 teams) and aren't refitted.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+      <c r="A4" s="23" t="inlineStr">
         <is>
           <t>Units</t>
         </is>
       </c>
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Win on a minus line = +1. Win on a plus line = line / 100 (e.g. +240 wins 2.4). Loss on a minus line = line / 100 (e.g. -240 loses 2.4). Loss on a plus line = -1. Results include overtime and the shootout.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t>Lines</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>From ESPN's free odds feed: DraftKings, or ESPN BET where DraftKings isn't listed. Oct 6-21, 2026 and all of 2025-26 use closing lines. From Oct 22, 2026, every game is picked 2 hours before the day's first game at the line right then, and units are graded on that line. A game without a line at that time gets its closing line, and the Line source column says so.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>Daily schedule</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Every morning after 6 am Central: last night's games are scored and graded, and the rule is reset. Two hours before the day's first game: every game is picked, this file is rebuilt and emailed.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>The daily rule</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Every rule of the form 'line from X to Y, differential from A up to B, home picks / away picks / either' is tried on every graded 2026-27 pick up to that morning, with every line and every differential seen so far as a possible cut point, and the one that would have made the most units wins (ties go to the rule with more bets). A bound at the edge of the lines seen so far is left open. 'Fits that day's rule' marks the picks it chose.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>Caution</t>
         </is>
       </c>
-      <c r="B8" s="18" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>The daily rule is the best fit to the past by construction, so its record always looks good. The honest test is the Dynamic Bet Results tab: only the picks that were emailed under each day's rule, before their games, at the line in the email. On 2025-26, rules found this way didn't carry over from one half of the season to the other or to 2026-27.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-21 22:50 CT.</t>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-21 22:51 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-22 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -6194,7 +6194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6279,6 +6279,38 @@
       </c>
       <c r="G4" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>46-18, +23.02 units</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>67-43, +12.17 units</t>
+        </is>
+      </c>
+      <c r="E5" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A5,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A5,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G5" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A5)</f>
         <v/>
       </c>
     </row>
@@ -65956,7 +65988,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-21 22:51 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-22 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-23 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -742,8 +742,16 @@
         <f>IF(AND(G9&lt;&gt;"W",G9&lt;&gt;"L"),"",IF(G9="W",IF(D9&gt;0,D9/100,1),IF(D9&lt;0,D9/100,-1)))</f>
         <v/>
       </c>
-      <c r="G9" s="11" t="inlineStr"/>
-      <c r="H9" s="10" t="inlineStr"/>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>NYR 4, TOR 5</t>
+        </is>
+      </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
@@ -774,8 +782,16 @@
         <f>IF(AND(G10&lt;&gt;"W",G10&lt;&gt;"L"),"",IF(G10="W",IF(D10&gt;0,D10/100,1),IF(D10&lt;0,D10/100,-1)))</f>
         <v/>
       </c>
-      <c r="G10" s="11" t="inlineStr"/>
-      <c r="H10" s="10" t="inlineStr"/>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>SJS 6, OTT 2</t>
+        </is>
+      </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
@@ -806,8 +822,16 @@
         <f>IF(AND(G11&lt;&gt;"W",G11&lt;&gt;"L"),"",IF(G11="W",IF(D11&gt;0,D11/100,1),IF(D11&lt;0,D11/100,-1)))</f>
         <v/>
       </c>
-      <c r="G11" s="11" t="inlineStr"/>
-      <c r="H11" s="10" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>FLA 0, PIT 4</t>
+        </is>
+      </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
@@ -838,8 +862,16 @@
         <f>IF(AND(G12&lt;&gt;"W",G12&lt;&gt;"L"),"",IF(G12="W",IF(D12&gt;0,D12/100,1),IF(D12&lt;0,D12/100,-1)))</f>
         <v/>
       </c>
-      <c r="G12" s="11" t="inlineStr"/>
-      <c r="H12" s="10" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>LAK 3, NYI 2</t>
+        </is>
+      </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
@@ -870,8 +902,16 @@
         <f>IF(AND(G13&lt;&gt;"W",G13&lt;&gt;"L"),"",IF(G13="W",IF(D13&gt;0,D13/100,1),IF(D13&lt;0,D13/100,-1)))</f>
         <v/>
       </c>
-      <c r="G13" s="11" t="inlineStr"/>
-      <c r="H13" s="10" t="inlineStr"/>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>VGK 2, STL 6</t>
+        </is>
+      </c>
       <c r="I13" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
@@ -902,8 +942,16 @@
         <f>IF(AND(G14&lt;&gt;"W",G14&lt;&gt;"L"),"",IF(G14="W",IF(D14&gt;0,D14/100,1),IF(D14&lt;0,D14/100,-1)))</f>
         <v/>
       </c>
-      <c r="G14" s="11" t="inlineStr"/>
-      <c r="H14" s="10" t="inlineStr"/>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>CAR 5, EDM 6</t>
+        </is>
+      </c>
       <c r="I14" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
@@ -934,8 +982,16 @@
         <f>IF(AND(G15&lt;&gt;"W",G15&lt;&gt;"L"),"",IF(G15="W",IF(D15&gt;0,D15/100,1),IF(D15&lt;0,D15/100,-1)))</f>
         <v/>
       </c>
-      <c r="G15" s="11" t="inlineStr"/>
-      <c r="H15" s="10" t="inlineStr"/>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>UTA 3, SEA 5</t>
+        </is>
+      </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
@@ -966,8 +1022,16 @@
         <f>IF(AND(G16&lt;&gt;"W",G16&lt;&gt;"L"),"",IF(G16="W",IF(D16&gt;0,D16/100,1),IF(D16&lt;0,D16/100,-1)))</f>
         <v/>
       </c>
-      <c r="G16" s="11" t="inlineStr"/>
-      <c r="H16" s="10" t="inlineStr"/>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>DET 5, VAN 2</t>
+        </is>
+      </c>
       <c r="I16" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
@@ -1036,7 +1100,7 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Today's rule: Bet the pick when it has a line from -192 to +110 and a differential of 23.51 or less; home or away.</t>
+          <t>Today's rule: Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
         </is>
       </c>
     </row>
@@ -6453,8 +6517,16 @@
         <f>IF(OR(F119="",G119="",AND(I119&lt;&gt;"W",I119&lt;&gt;"L")),"",IF(I119="W",IF(G119&gt;0,G119/100,1),IF(G119&lt;0,G119/100,-1)))</f>
         <v/>
       </c>
-      <c r="I119" s="11" t="inlineStr"/>
-      <c r="J119" s="10" t="inlineStr"/>
+      <c r="I119" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J119" s="10" t="inlineStr">
+        <is>
+          <t>NSH 0, BOS 6</t>
+        </is>
+      </c>
       <c r="K119" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6497,8 +6569,16 @@
         <f>IF(OR(F120="",G120="",AND(I120&lt;&gt;"W",I120&lt;&gt;"L")),"",IF(I120="W",IF(G120&gt;0,G120/100,1),IF(G120&lt;0,G120/100,-1)))</f>
         <v/>
       </c>
-      <c r="I120" s="11" t="inlineStr"/>
-      <c r="J120" s="10" t="inlineStr"/>
+      <c r="I120" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J120" s="10" t="inlineStr">
+        <is>
+          <t>NYR 4, TOR 5</t>
+        </is>
+      </c>
       <c r="K120" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6541,8 +6621,16 @@
         <f>IF(OR(F121="",G121="",AND(I121&lt;&gt;"W",I121&lt;&gt;"L")),"",IF(I121="W",IF(G121&gt;0,G121/100,1),IF(G121&lt;0,G121/100,-1)))</f>
         <v/>
       </c>
-      <c r="I121" s="11" t="inlineStr"/>
-      <c r="J121" s="10" t="inlineStr"/>
+      <c r="I121" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J121" s="10" t="inlineStr">
+        <is>
+          <t>SJS 6, OTT 2</t>
+        </is>
+      </c>
       <c r="K121" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6585,8 +6673,16 @@
         <f>IF(OR(F122="",G122="",AND(I122&lt;&gt;"W",I122&lt;&gt;"L")),"",IF(I122="W",IF(G122&gt;0,G122/100,1),IF(G122&lt;0,G122/100,-1)))</f>
         <v/>
       </c>
-      <c r="I122" s="11" t="inlineStr"/>
-      <c r="J122" s="10" t="inlineStr"/>
+      <c r="I122" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J122" s="10" t="inlineStr">
+        <is>
+          <t>ANA 1, NJD 4</t>
+        </is>
+      </c>
       <c r="K122" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6629,8 +6725,16 @@
         <f>IF(OR(F123="",G123="",AND(I123&lt;&gt;"W",I123&lt;&gt;"L")),"",IF(I123="W",IF(G123&gt;0,G123/100,1),IF(G123&lt;0,G123/100,-1)))</f>
         <v/>
       </c>
-      <c r="I123" s="11" t="inlineStr"/>
-      <c r="J123" s="10" t="inlineStr"/>
+      <c r="I123" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J123" s="10" t="inlineStr">
+        <is>
+          <t>FLA 0, PIT 4</t>
+        </is>
+      </c>
       <c r="K123" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6673,8 +6777,16 @@
         <f>IF(OR(F124="",G124="",AND(I124&lt;&gt;"W",I124&lt;&gt;"L")),"",IF(I124="W",IF(G124&gt;0,G124/100,1),IF(G124&lt;0,G124/100,-1)))</f>
         <v/>
       </c>
-      <c r="I124" s="11" t="inlineStr"/>
-      <c r="J124" s="10" t="inlineStr"/>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J124" s="10" t="inlineStr">
+        <is>
+          <t>LAK 3, NYI 2</t>
+        </is>
+      </c>
       <c r="K124" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6717,8 +6829,16 @@
         <f>IF(OR(F125="",G125="",AND(I125&lt;&gt;"W",I125&lt;&gt;"L")),"",IF(I125="W",IF(G125&gt;0,G125/100,1),IF(G125&lt;0,G125/100,-1)))</f>
         <v/>
       </c>
-      <c r="I125" s="11" t="inlineStr"/>
-      <c r="J125" s="10" t="inlineStr"/>
+      <c r="I125" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J125" s="10" t="inlineStr">
+        <is>
+          <t>VGK 2, STL 6</t>
+        </is>
+      </c>
       <c r="K125" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6761,8 +6881,16 @@
         <f>IF(OR(F126="",G126="",AND(I126&lt;&gt;"W",I126&lt;&gt;"L")),"",IF(I126="W",IF(G126&gt;0,G126/100,1),IF(G126&lt;0,G126/100,-1)))</f>
         <v/>
       </c>
-      <c r="I126" s="11" t="inlineStr"/>
-      <c r="J126" s="10" t="inlineStr"/>
+      <c r="I126" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J126" s="10" t="inlineStr">
+        <is>
+          <t>WPG 2, DAL 3</t>
+        </is>
+      </c>
       <c r="K126" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6805,8 +6933,16 @@
         <f>IF(OR(F127="",G127="",AND(I127&lt;&gt;"W",I127&lt;&gt;"L")),"",IF(I127="W",IF(G127&gt;0,G127/100,1),IF(G127&lt;0,G127/100,-1)))</f>
         <v/>
       </c>
-      <c r="I127" s="11" t="inlineStr"/>
-      <c r="J127" s="10" t="inlineStr"/>
+      <c r="I127" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J127" s="10" t="inlineStr">
+        <is>
+          <t>MIN 1, CGY 2</t>
+        </is>
+      </c>
       <c r="K127" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6849,8 +6985,16 @@
         <f>IF(OR(F128="",G128="",AND(I128&lt;&gt;"W",I128&lt;&gt;"L")),"",IF(I128="W",IF(G128&gt;0,G128/100,1),IF(G128&lt;0,G128/100,-1)))</f>
         <v/>
       </c>
-      <c r="I128" s="11" t="inlineStr"/>
-      <c r="J128" s="10" t="inlineStr"/>
+      <c r="I128" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J128" s="10" t="inlineStr">
+        <is>
+          <t>CAR 5, EDM 6</t>
+        </is>
+      </c>
       <c r="K128" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6893,8 +7037,16 @@
         <f>IF(OR(F129="",G129="",AND(I129&lt;&gt;"W",I129&lt;&gt;"L")),"",IF(I129="W",IF(G129&gt;0,G129/100,1),IF(G129&lt;0,G129/100,-1)))</f>
         <v/>
       </c>
-      <c r="I129" s="11" t="inlineStr"/>
-      <c r="J129" s="10" t="inlineStr"/>
+      <c r="I129" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J129" s="10" t="inlineStr">
+        <is>
+          <t>UTA 3, SEA 5</t>
+        </is>
+      </c>
       <c r="K129" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6937,8 +7089,16 @@
         <f>IF(OR(F130="",G130="",AND(I130&lt;&gt;"W",I130&lt;&gt;"L")),"",IF(I130="W",IF(G130&gt;0,G130/100,1),IF(G130&lt;0,G130/100,-1)))</f>
         <v/>
       </c>
-      <c r="I130" s="11" t="inlineStr"/>
-      <c r="J130" s="10" t="inlineStr"/>
+      <c r="I130" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J130" s="10" t="inlineStr">
+        <is>
+          <t>DET 5, VAN 2</t>
+        </is>
+      </c>
       <c r="K130" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -6978,7 +7138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7095,6 +7255,38 @@
       </c>
       <c r="G5" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>54-23, +20.97 units</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>72-50, +7.82 units</t>
+        </is>
+      </c>
+      <c r="E6" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A6,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A6,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G6" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A6)</f>
         <v/>
       </c>
     </row>
@@ -66772,7 +66964,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-22 16:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-23 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-23 17:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$132</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1066,7 +1066,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1128,19 +1128,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H130)</f>
+        <f>SUM(H9:H132)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I130,"W")/(COUNTIF(I9:I130,"W")+COUNTIF(I9:I130,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I132,"W")/(COUNTIF(I9:I132,"W")+COUNTIF(I9:I132,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I130,"W")&amp;"-"&amp;COUNTIF(I9:I130,"L")</f>
+        <f>COUNTIF(I9:I132,"W")&amp;"-"&amp;COUNTIF(I9:I132,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I130,"W")+COUNTIF(I9:I130,"L")</f>
+        <f>COUNTIF(I9:I132,"W")+COUNTIF(I9:I132,"L")</f>
         <v/>
       </c>
     </row>
@@ -7110,8 +7110,92 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="9" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B131" s="10" t="inlineStr">
+        <is>
+          <t>MTL @ CHI</t>
+        </is>
+      </c>
+      <c r="C131" s="13" t="n">
+        <v>76.81</v>
+      </c>
+      <c r="D131" s="13" t="n">
+        <v>54.49</v>
+      </c>
+      <c r="E131" s="13">
+        <f>IF(OR(C131="",D131=""),"",ABS(C131-D131))</f>
+        <v/>
+      </c>
+      <c r="F131" s="11" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="G131" s="12" t="n"/>
+      <c r="H131" s="14">
+        <f>IF(OR(F131="",G131="",AND(I131&lt;&gt;"W",I131&lt;&gt;"L")),"",IF(I131="W",IF(G131&gt;0,G131/100,1),IF(G131&lt;0,G131/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I131" s="11" t="inlineStr"/>
+      <c r="J131" s="10" t="inlineStr"/>
+      <c r="K131" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L131" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="9" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B132" s="10" t="inlineStr">
+        <is>
+          <t>TBL @ COL</t>
+        </is>
+      </c>
+      <c r="C132" s="13" t="n">
+        <v>81.48</v>
+      </c>
+      <c r="D132" s="13" t="n">
+        <v>69.5</v>
+      </c>
+      <c r="E132" s="13">
+        <f>IF(OR(C132="",D132=""),"",ABS(C132-D132))</f>
+        <v/>
+      </c>
+      <c r="F132" s="11" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="G132" s="12" t="n"/>
+      <c r="H132" s="14">
+        <f>IF(OR(F132="",G132="",AND(I132&lt;&gt;"W",I132&lt;&gt;"L")),"",IF(I132="W",IF(G132&gt;0,G132/100,1),IF(G132&lt;0,G132/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I132" s="11" t="inlineStr"/>
+      <c r="J132" s="10" t="inlineStr"/>
+      <c r="K132" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L132" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L130"/>
+  <autoFilter ref="A8:L132"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -7120,7 +7204,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H130">
+  <conditionalFormatting sqref="H9:H132">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -66964,7 +67048,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-23 06:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-23 17:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-24 06:15 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -7139,8 +7139,16 @@
         <f>IF(OR(F131="",G131="",AND(I131&lt;&gt;"W",I131&lt;&gt;"L")),"",IF(I131="W",IF(G131&gt;0,G131/100,1),IF(G131&lt;0,G131/100,-1)))</f>
         <v/>
       </c>
-      <c r="I131" s="11" t="inlineStr"/>
-      <c r="J131" s="10" t="inlineStr"/>
+      <c r="I131" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J131" s="10" t="inlineStr">
+        <is>
+          <t>MTL 4, CHI 1</t>
+        </is>
+      </c>
       <c r="K131" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -7181,8 +7189,16 @@
         <f>IF(OR(F132="",G132="",AND(I132&lt;&gt;"W",I132&lt;&gt;"L")),"",IF(I132="W",IF(G132&gt;0,G132/100,1),IF(G132&lt;0,G132/100,-1)))</f>
         <v/>
       </c>
-      <c r="I132" s="11" t="inlineStr"/>
-      <c r="J132" s="10" t="inlineStr"/>
+      <c r="I132" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J132" s="10" t="inlineStr">
+        <is>
+          <t>TBL 3, COL 6</t>
+        </is>
+      </c>
       <c r="K132" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -7222,7 +7238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7371,6 +7387,38 @@
       </c>
       <c r="G6" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>54-23, +20.97 units</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>72-50, +7.82 units</t>
+        </is>
+      </c>
+      <c r="E7" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A7,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A7,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G7" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A7)</f>
         <v/>
       </c>
     </row>
@@ -67048,7 +67096,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-23 17:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-24 06:15 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-24 10:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$144</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -651,23 +651,23 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(F9:F16)</f>
+        <f>SUM(F9:F22)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(G9:G16,"W")/(COUNTIF(G9:G16,"W")+COUNTIF(G9:G16,"L")),"")</f>
+        <f>IFERROR(COUNTIF(G9:G22,"W")/(COUNTIF(G9:G22,"W")+COUNTIF(G9:G22,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(G9:G16,"W")&amp;"-"&amp;COUNTIF(G9:G16,"L")</f>
+        <f>COUNTIF(G9:G22,"W")&amp;"-"&amp;COUNTIF(G9:G22,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(G9:G16,"W")+COUNTIF(G9:G16,"L")</f>
+        <f>COUNTIF(G9:G22,"W")+COUNTIF(G9:G22,"L")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTA(B9:B16)-COUNTIF(G9:G16,"W")-COUNTIF(G9:G16,"L")</f>
+        <f>COUNTA(B9:B22)-COUNTIF(G9:G22,"W")-COUNTIF(G9:G22,"L")</f>
         <v/>
       </c>
     </row>
@@ -1038,8 +1038,200 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>ANA @ PHI</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>-122</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="F17" s="14">
+        <f>IF(AND(G17&lt;&gt;"W",G17&lt;&gt;"L"),"",IF(G17="W",IF(D17&gt;0,D17/100,1),IF(D17&lt;0,D17/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G17" s="11" t="inlineStr"/>
+      <c r="H17" s="10" t="inlineStr"/>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>LAK @ NJD</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>-192</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="F18" s="14">
+        <f>IF(AND(G18&lt;&gt;"W",G18&lt;&gt;"L"),"",IF(G18="W",IF(D18&gt;0,D18/100,1),IF(D18&lt;0,D18/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G18" s="11" t="inlineStr"/>
+      <c r="H18" s="10" t="inlineStr"/>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>NYR @ OTT</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>-125</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>11.62</v>
+      </c>
+      <c r="F19" s="14">
+        <f>IF(AND(G19&lt;&gt;"W",G19&lt;&gt;"L"),"",IF(G19="W",IF(D19&gt;0,D19/100,1),IF(D19&lt;0,D19/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G19" s="11" t="inlineStr"/>
+      <c r="H19" s="10" t="inlineStr"/>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>BUF @ WSH</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>-125</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="F20" s="14">
+        <f>IF(AND(G20&lt;&gt;"W",G20&lt;&gt;"L"),"",IF(G20="W",IF(D20&gt;0,D20/100,1),IF(D20&lt;0,D20/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G20" s="11" t="inlineStr"/>
+      <c r="H20" s="10" t="inlineStr"/>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>TBL @ UTA</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>-142</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="F21" s="14">
+        <f>IF(AND(G21&lt;&gt;"W",G21&lt;&gt;"L"),"",IF(G21="W",IF(D21&gt;0,D21/100,1),IF(D21&lt;0,D21/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G21" s="11" t="inlineStr"/>
+      <c r="H21" s="10" t="inlineStr"/>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>MIN @ SEA</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>-155</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>7.91</v>
+      </c>
+      <c r="F22" s="14">
+        <f>IF(AND(G22&lt;&gt;"W",G22&lt;&gt;"L"),"",IF(G22="W",IF(D22&gt;0,D22/100,1),IF(D22&lt;0,D22/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G22" s="11" t="inlineStr"/>
+      <c r="H22" s="10" t="inlineStr"/>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:I16"/>
+  <autoFilter ref="A8:I22"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -1048,7 +1240,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F16">
+  <conditionalFormatting sqref="F9:F22">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -1066,7 +1258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1128,19 +1320,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H132)</f>
+        <f>SUM(H9:H144)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I132,"W")/(COUNTIF(I9:I132,"W")+COUNTIF(I9:I132,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I144,"W")/(COUNTIF(I9:I144,"W")+COUNTIF(I9:I144,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I132,"W")&amp;"-"&amp;COUNTIF(I9:I132,"L")</f>
+        <f>COUNTIF(I9:I144,"W")&amp;"-"&amp;COUNTIF(I9:I144,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I132,"W")+COUNTIF(I9:I132,"L")</f>
+        <f>COUNTIF(I9:I144,"W")+COUNTIF(I9:I144,"L")</f>
         <v/>
       </c>
     </row>
@@ -7210,8 +7402,536 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B133" s="10" t="inlineStr">
+        <is>
+          <t>ANA @ PHI</t>
+        </is>
+      </c>
+      <c r="C133" s="13" t="n">
+        <v>59.46</v>
+      </c>
+      <c r="D133" s="13" t="n">
+        <v>76.19</v>
+      </c>
+      <c r="E133" s="13">
+        <f>IF(OR(C133="",D133=""),"",ABS(C133-D133))</f>
+        <v/>
+      </c>
+      <c r="F133" s="11" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="G133" s="12" t="n">
+        <v>-122</v>
+      </c>
+      <c r="H133" s="14">
+        <f>IF(OR(F133="",G133="",AND(I133&lt;&gt;"W",I133&lt;&gt;"L")),"",IF(I133="W",IF(G133&gt;0,G133/100,1),IF(G133&lt;0,G133/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I133" s="11" t="inlineStr"/>
+      <c r="J133" s="10" t="inlineStr"/>
+      <c r="K133" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L133" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B134" s="10" t="inlineStr">
+        <is>
+          <t>LAK @ NJD</t>
+        </is>
+      </c>
+      <c r="C134" s="13" t="n">
+        <v>71.5</v>
+      </c>
+      <c r="D134" s="13" t="n">
+        <v>80.54000000000001</v>
+      </c>
+      <c r="E134" s="13">
+        <f>IF(OR(C134="",D134=""),"",ABS(C134-D134))</f>
+        <v/>
+      </c>
+      <c r="F134" s="11" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="G134" s="12" t="n">
+        <v>-192</v>
+      </c>
+      <c r="H134" s="14">
+        <f>IF(OR(F134="",G134="",AND(I134&lt;&gt;"W",I134&lt;&gt;"L")),"",IF(I134="W",IF(G134&gt;0,G134/100,1),IF(G134&lt;0,G134/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I134" s="11" t="inlineStr"/>
+      <c r="J134" s="10" t="inlineStr"/>
+      <c r="K134" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L134" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B135" s="10" t="inlineStr">
+        <is>
+          <t>SJS @ BOS</t>
+        </is>
+      </c>
+      <c r="C135" s="13" t="n">
+        <v>64.26000000000001</v>
+      </c>
+      <c r="D135" s="13" t="n">
+        <v>91.76000000000001</v>
+      </c>
+      <c r="E135" s="13">
+        <f>IF(OR(C135="",D135=""),"",ABS(C135-D135))</f>
+        <v/>
+      </c>
+      <c r="F135" s="11" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="G135" s="12" t="n">
+        <v>-192</v>
+      </c>
+      <c r="H135" s="14">
+        <f>IF(OR(F135="",G135="",AND(I135&lt;&gt;"W",I135&lt;&gt;"L")),"",IF(I135="W",IF(G135&gt;0,G135/100,1),IF(G135&lt;0,G135/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I135" s="11" t="inlineStr"/>
+      <c r="J135" s="10" t="inlineStr"/>
+      <c r="K135" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L135" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B136" s="10" t="inlineStr">
+        <is>
+          <t>NYR @ OTT</t>
+        </is>
+      </c>
+      <c r="C136" s="13" t="n">
+        <v>64.12</v>
+      </c>
+      <c r="D136" s="13" t="n">
+        <v>75.73999999999999</v>
+      </c>
+      <c r="E136" s="13">
+        <f>IF(OR(C136="",D136=""),"",ABS(C136-D136))</f>
+        <v/>
+      </c>
+      <c r="F136" s="11" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="G136" s="12" t="n">
+        <v>-125</v>
+      </c>
+      <c r="H136" s="14">
+        <f>IF(OR(F136="",G136="",AND(I136&lt;&gt;"W",I136&lt;&gt;"L")),"",IF(I136="W",IF(G136&gt;0,G136/100,1),IF(G136&lt;0,G136/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I136" s="11" t="inlineStr"/>
+      <c r="J136" s="10" t="inlineStr"/>
+      <c r="K136" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L136" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B137" s="10" t="inlineStr">
+        <is>
+          <t>NSH @ PIT</t>
+        </is>
+      </c>
+      <c r="C137" s="13" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="D137" s="13" t="n">
+        <v>79.58</v>
+      </c>
+      <c r="E137" s="13">
+        <f>IF(OR(C137="",D137=""),"",ABS(C137-D137))</f>
+        <v/>
+      </c>
+      <c r="F137" s="11" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="G137" s="12" t="n">
+        <v>-142</v>
+      </c>
+      <c r="H137" s="14">
+        <f>IF(OR(F137="",G137="",AND(I137&lt;&gt;"W",I137&lt;&gt;"L")),"",IF(I137="W",IF(G137&gt;0,G137/100,1),IF(G137&lt;0,G137/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I137" s="11" t="inlineStr"/>
+      <c r="J137" s="10" t="inlineStr"/>
+      <c r="K137" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L137" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B138" s="10" t="inlineStr">
+        <is>
+          <t>BUF @ WSH</t>
+        </is>
+      </c>
+      <c r="C138" s="13" t="n">
+        <v>63.81</v>
+      </c>
+      <c r="D138" s="13" t="n">
+        <v>71.28</v>
+      </c>
+      <c r="E138" s="13">
+        <f>IF(OR(C138="",D138=""),"",ABS(C138-D138))</f>
+        <v/>
+      </c>
+      <c r="F138" s="11" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="G138" s="12" t="n">
+        <v>-125</v>
+      </c>
+      <c r="H138" s="14">
+        <f>IF(OR(F138="",G138="",AND(I138&lt;&gt;"W",I138&lt;&gt;"L")),"",IF(I138="W",IF(G138&gt;0,G138/100,1),IF(G138&lt;0,G138/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I138" s="11" t="inlineStr"/>
+      <c r="J138" s="10" t="inlineStr"/>
+      <c r="K138" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L138" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B139" s="10" t="inlineStr">
+        <is>
+          <t>VGK @ CBJ</t>
+        </is>
+      </c>
+      <c r="C139" s="13" t="n">
+        <v>60.92</v>
+      </c>
+      <c r="D139" s="13" t="n">
+        <v>63.32</v>
+      </c>
+      <c r="E139" s="13">
+        <f>IF(OR(C139="",D139=""),"",ABS(C139-D139))</f>
+        <v/>
+      </c>
+      <c r="F139" s="11" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="G139" s="12" t="n">
+        <v>120</v>
+      </c>
+      <c r="H139" s="14">
+        <f>IF(OR(F139="",G139="",AND(I139&lt;&gt;"W",I139&lt;&gt;"L")),"",IF(I139="W",IF(G139&gt;0,G139/100,1),IF(G139&lt;0,G139/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I139" s="11" t="inlineStr"/>
+      <c r="J139" s="10" t="inlineStr"/>
+      <c r="K139" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L139" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B140" s="10" t="inlineStr">
+        <is>
+          <t>CAR @ STL</t>
+        </is>
+      </c>
+      <c r="C140" s="13" t="n">
+        <v>74.08</v>
+      </c>
+      <c r="D140" s="13" t="n">
+        <v>79.08</v>
+      </c>
+      <c r="E140" s="13">
+        <f>IF(OR(C140="",D140=""),"",ABS(C140-D140))</f>
+        <v/>
+      </c>
+      <c r="F140" s="11" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="G140" s="12" t="n">
+        <v>130</v>
+      </c>
+      <c r="H140" s="14">
+        <f>IF(OR(F140="",G140="",AND(I140&lt;&gt;"W",I140&lt;&gt;"L")),"",IF(I140="W",IF(G140&gt;0,G140/100,1),IF(G140&lt;0,G140/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I140" s="11" t="inlineStr"/>
+      <c r="J140" s="10" t="inlineStr"/>
+      <c r="K140" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L140" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B141" s="10" t="inlineStr">
+        <is>
+          <t>TOR @ EDM</t>
+        </is>
+      </c>
+      <c r="C141" s="13" t="n">
+        <v>75.88</v>
+      </c>
+      <c r="D141" s="13" t="n">
+        <v>65.92</v>
+      </c>
+      <c r="E141" s="13">
+        <f>IF(OR(C141="",D141=""),"",ABS(C141-D141))</f>
+        <v/>
+      </c>
+      <c r="F141" s="11" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="G141" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="H141" s="14">
+        <f>IF(OR(F141="",G141="",AND(I141&lt;&gt;"W",I141&lt;&gt;"L")),"",IF(I141="W",IF(G141&gt;0,G141/100,1),IF(G141&lt;0,G141/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I141" s="11" t="inlineStr"/>
+      <c r="J141" s="10" t="inlineStr"/>
+      <c r="K141" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L141" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B142" s="10" t="inlineStr">
+        <is>
+          <t>TBL @ UTA</t>
+        </is>
+      </c>
+      <c r="C142" s="13" t="n">
+        <v>71.16</v>
+      </c>
+      <c r="D142" s="13" t="n">
+        <v>74.02</v>
+      </c>
+      <c r="E142" s="13">
+        <f>IF(OR(C142="",D142=""),"",ABS(C142-D142))</f>
+        <v/>
+      </c>
+      <c r="F142" s="11" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="G142" s="12" t="n">
+        <v>-142</v>
+      </c>
+      <c r="H142" s="14">
+        <f>IF(OR(F142="",G142="",AND(I142&lt;&gt;"W",I142&lt;&gt;"L")),"",IF(I142="W",IF(G142&gt;0,G142/100,1),IF(G142&lt;0,G142/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I142" s="11" t="inlineStr"/>
+      <c r="J142" s="10" t="inlineStr"/>
+      <c r="K142" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L142" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B143" s="10" t="inlineStr">
+        <is>
+          <t>DET @ CGY</t>
+        </is>
+      </c>
+      <c r="C143" s="13" t="n">
+        <v>93.63</v>
+      </c>
+      <c r="D143" s="13" t="n">
+        <v>66.11</v>
+      </c>
+      <c r="E143" s="13">
+        <f>IF(OR(C143="",D143=""),"",ABS(C143-D143))</f>
+        <v/>
+      </c>
+      <c r="F143" s="11" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="G143" s="12" t="n">
+        <v>-148</v>
+      </c>
+      <c r="H143" s="14">
+        <f>IF(OR(F143="",G143="",AND(I143&lt;&gt;"W",I143&lt;&gt;"L")),"",IF(I143="W",IF(G143&gt;0,G143/100,1),IF(G143&lt;0,G143/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I143" s="11" t="inlineStr"/>
+      <c r="J143" s="10" t="inlineStr"/>
+      <c r="K143" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L143" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="9" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B144" s="10" t="inlineStr">
+        <is>
+          <t>MIN @ SEA</t>
+        </is>
+      </c>
+      <c r="C144" s="13" t="n">
+        <v>73.89</v>
+      </c>
+      <c r="D144" s="13" t="n">
+        <v>65.98</v>
+      </c>
+      <c r="E144" s="13">
+        <f>IF(OR(C144="",D144=""),"",ABS(C144-D144))</f>
+        <v/>
+      </c>
+      <c r="F144" s="11" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="G144" s="12" t="n">
+        <v>-155</v>
+      </c>
+      <c r="H144" s="14">
+        <f>IF(OR(F144="",G144="",AND(I144&lt;&gt;"W",I144&lt;&gt;"L")),"",IF(I144="W",IF(G144&gt;0,G144/100,1),IF(G144&lt;0,G144/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I144" s="11" t="inlineStr"/>
+      <c r="J144" s="10" t="inlineStr"/>
+      <c r="K144" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (10:00 AM CT)</t>
+        </is>
+      </c>
+      <c r="L144" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L132"/>
+  <autoFilter ref="A8:L144"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -7220,7 +7940,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H132">
+  <conditionalFormatting sqref="H9:H144">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -67096,7 +67816,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-24 06:15 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-24 10:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-25 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -1062,8 +1062,16 @@
         <f>IF(AND(G17&lt;&gt;"W",G17&lt;&gt;"L"),"",IF(G17="W",IF(D17&gt;0,D17/100,1),IF(D17&lt;0,D17/100,-1)))</f>
         <v/>
       </c>
-      <c r="G17" s="11" t="inlineStr"/>
-      <c r="H17" s="10" t="inlineStr"/>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>ANA 5, PHI 4</t>
+        </is>
+      </c>
       <c r="I17" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
@@ -1094,8 +1102,16 @@
         <f>IF(AND(G18&lt;&gt;"W",G18&lt;&gt;"L"),"",IF(G18="W",IF(D18&gt;0,D18/100,1),IF(D18&lt;0,D18/100,-1)))</f>
         <v/>
       </c>
-      <c r="G18" s="11" t="inlineStr"/>
-      <c r="H18" s="10" t="inlineStr"/>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>LAK 1, NJD 3</t>
+        </is>
+      </c>
       <c r="I18" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
@@ -1126,8 +1142,16 @@
         <f>IF(AND(G19&lt;&gt;"W",G19&lt;&gt;"L"),"",IF(G19="W",IF(D19&gt;0,D19/100,1),IF(D19&lt;0,D19/100,-1)))</f>
         <v/>
       </c>
-      <c r="G19" s="11" t="inlineStr"/>
-      <c r="H19" s="10" t="inlineStr"/>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>NYR 4, OTT 7</t>
+        </is>
+      </c>
       <c r="I19" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
@@ -1158,8 +1182,16 @@
         <f>IF(AND(G20&lt;&gt;"W",G20&lt;&gt;"L"),"",IF(G20="W",IF(D20&gt;0,D20/100,1),IF(D20&lt;0,D20/100,-1)))</f>
         <v/>
       </c>
-      <c r="G20" s="11" t="inlineStr"/>
-      <c r="H20" s="10" t="inlineStr"/>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>BUF 3, WSH 4</t>
+        </is>
+      </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
@@ -1190,8 +1222,16 @@
         <f>IF(AND(G21&lt;&gt;"W",G21&lt;&gt;"L"),"",IF(G21="W",IF(D21&gt;0,D21/100,1),IF(D21&lt;0,D21/100,-1)))</f>
         <v/>
       </c>
-      <c r="G21" s="11" t="inlineStr"/>
-      <c r="H21" s="10" t="inlineStr"/>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>TBL 4, UTA 5</t>
+        </is>
+      </c>
       <c r="I21" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
@@ -1222,8 +1262,16 @@
         <f>IF(AND(G22&lt;&gt;"W",G22&lt;&gt;"L"),"",IF(G22="W",IF(D22&gt;0,D22/100,1),IF(D22&lt;0,D22/100,-1)))</f>
         <v/>
       </c>
-      <c r="G22" s="11" t="inlineStr"/>
-      <c r="H22" s="10" t="inlineStr"/>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>MIN 5, SEA 1</t>
+        </is>
+      </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
@@ -1292,7 +1340,7 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Today's rule: Bet the pick when it has any line up to +110 and a differential of 19.38 or less; home or away.</t>
+          <t>Today's rule: Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
         </is>
       </c>
     </row>
@@ -7433,8 +7481,16 @@
         <f>IF(OR(F133="",G133="",AND(I133&lt;&gt;"W",I133&lt;&gt;"L")),"",IF(I133="W",IF(G133&gt;0,G133/100,1),IF(G133&lt;0,G133/100,-1)))</f>
         <v/>
       </c>
-      <c r="I133" s="11" t="inlineStr"/>
-      <c r="J133" s="10" t="inlineStr"/>
+      <c r="I133" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J133" s="10" t="inlineStr">
+        <is>
+          <t>ANA 5, PHI 4</t>
+        </is>
+      </c>
       <c r="K133" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7477,8 +7533,16 @@
         <f>IF(OR(F134="",G134="",AND(I134&lt;&gt;"W",I134&lt;&gt;"L")),"",IF(I134="W",IF(G134&gt;0,G134/100,1),IF(G134&lt;0,G134/100,-1)))</f>
         <v/>
       </c>
-      <c r="I134" s="11" t="inlineStr"/>
-      <c r="J134" s="10" t="inlineStr"/>
+      <c r="I134" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J134" s="10" t="inlineStr">
+        <is>
+          <t>LAK 1, NJD 3</t>
+        </is>
+      </c>
       <c r="K134" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7521,8 +7585,16 @@
         <f>IF(OR(F135="",G135="",AND(I135&lt;&gt;"W",I135&lt;&gt;"L")),"",IF(I135="W",IF(G135&gt;0,G135/100,1),IF(G135&lt;0,G135/100,-1)))</f>
         <v/>
       </c>
-      <c r="I135" s="11" t="inlineStr"/>
-      <c r="J135" s="10" t="inlineStr"/>
+      <c r="I135" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J135" s="10" t="inlineStr">
+        <is>
+          <t>SJS 4, BOS 6</t>
+        </is>
+      </c>
       <c r="K135" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7565,8 +7637,16 @@
         <f>IF(OR(F136="",G136="",AND(I136&lt;&gt;"W",I136&lt;&gt;"L")),"",IF(I136="W",IF(G136&gt;0,G136/100,1),IF(G136&lt;0,G136/100,-1)))</f>
         <v/>
       </c>
-      <c r="I136" s="11" t="inlineStr"/>
-      <c r="J136" s="10" t="inlineStr"/>
+      <c r="I136" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J136" s="10" t="inlineStr">
+        <is>
+          <t>NYR 4, OTT 7</t>
+        </is>
+      </c>
       <c r="K136" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7609,8 +7689,16 @@
         <f>IF(OR(F137="",G137="",AND(I137&lt;&gt;"W",I137&lt;&gt;"L")),"",IF(I137="W",IF(G137&gt;0,G137/100,1),IF(G137&lt;0,G137/100,-1)))</f>
         <v/>
       </c>
-      <c r="I137" s="11" t="inlineStr"/>
-      <c r="J137" s="10" t="inlineStr"/>
+      <c r="I137" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J137" s="10" t="inlineStr">
+        <is>
+          <t>NSH 2, PIT 3</t>
+        </is>
+      </c>
       <c r="K137" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7653,8 +7741,16 @@
         <f>IF(OR(F138="",G138="",AND(I138&lt;&gt;"W",I138&lt;&gt;"L")),"",IF(I138="W",IF(G138&gt;0,G138/100,1),IF(G138&lt;0,G138/100,-1)))</f>
         <v/>
       </c>
-      <c r="I138" s="11" t="inlineStr"/>
-      <c r="J138" s="10" t="inlineStr"/>
+      <c r="I138" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J138" s="10" t="inlineStr">
+        <is>
+          <t>BUF 3, WSH 4</t>
+        </is>
+      </c>
       <c r="K138" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7697,8 +7793,16 @@
         <f>IF(OR(F139="",G139="",AND(I139&lt;&gt;"W",I139&lt;&gt;"L")),"",IF(I139="W",IF(G139&gt;0,G139/100,1),IF(G139&lt;0,G139/100,-1)))</f>
         <v/>
       </c>
-      <c r="I139" s="11" t="inlineStr"/>
-      <c r="J139" s="10" t="inlineStr"/>
+      <c r="I139" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J139" s="10" t="inlineStr">
+        <is>
+          <t>VGK 1, CBJ 2</t>
+        </is>
+      </c>
       <c r="K139" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7741,8 +7845,16 @@
         <f>IF(OR(F140="",G140="",AND(I140&lt;&gt;"W",I140&lt;&gt;"L")),"",IF(I140="W",IF(G140&gt;0,G140/100,1),IF(G140&lt;0,G140/100,-1)))</f>
         <v/>
       </c>
-      <c r="I140" s="11" t="inlineStr"/>
-      <c r="J140" s="10" t="inlineStr"/>
+      <c r="I140" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J140" s="10" t="inlineStr">
+        <is>
+          <t>CAR 4, STL 0</t>
+        </is>
+      </c>
       <c r="K140" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7785,8 +7897,16 @@
         <f>IF(OR(F141="",G141="",AND(I141&lt;&gt;"W",I141&lt;&gt;"L")),"",IF(I141="W",IF(G141&gt;0,G141/100,1),IF(G141&lt;0,G141/100,-1)))</f>
         <v/>
       </c>
-      <c r="I141" s="11" t="inlineStr"/>
-      <c r="J141" s="10" t="inlineStr"/>
+      <c r="I141" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J141" s="10" t="inlineStr">
+        <is>
+          <t>TOR 7, EDM 2</t>
+        </is>
+      </c>
       <c r="K141" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7829,8 +7949,16 @@
         <f>IF(OR(F142="",G142="",AND(I142&lt;&gt;"W",I142&lt;&gt;"L")),"",IF(I142="W",IF(G142&gt;0,G142/100,1),IF(G142&lt;0,G142/100,-1)))</f>
         <v/>
       </c>
-      <c r="I142" s="11" t="inlineStr"/>
-      <c r="J142" s="10" t="inlineStr"/>
+      <c r="I142" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J142" s="10" t="inlineStr">
+        <is>
+          <t>TBL 4, UTA 5</t>
+        </is>
+      </c>
       <c r="K142" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7873,8 +8001,16 @@
         <f>IF(OR(F143="",G143="",AND(I143&lt;&gt;"W",I143&lt;&gt;"L")),"",IF(I143="W",IF(G143&gt;0,G143/100,1),IF(G143&lt;0,G143/100,-1)))</f>
         <v/>
       </c>
-      <c r="I143" s="11" t="inlineStr"/>
-      <c r="J143" s="10" t="inlineStr"/>
+      <c r="I143" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J143" s="10" t="inlineStr">
+        <is>
+          <t>DET 1, CGY 4</t>
+        </is>
+      </c>
       <c r="K143" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7917,8 +8053,16 @@
         <f>IF(OR(F144="",G144="",AND(I144&lt;&gt;"W",I144&lt;&gt;"L")),"",IF(I144="W",IF(G144&gt;0,G144/100,1),IF(G144&lt;0,G144/100,-1)))</f>
         <v/>
       </c>
-      <c r="I144" s="11" t="inlineStr"/>
-      <c r="J144" s="10" t="inlineStr"/>
+      <c r="I144" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J144" s="10" t="inlineStr">
+        <is>
+          <t>MIN 5, SEA 1</t>
+        </is>
+      </c>
       <c r="K144" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (10:00 AM CT)</t>
@@ -7958,7 +8102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8139,6 +8283,38 @@
       </c>
       <c r="G7" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>48-19, +27.21 units</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>81-53, +13.82 units</t>
+        </is>
+      </c>
+      <c r="E8" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A8,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A8,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G8" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A8)</f>
         <v/>
       </c>
     </row>
@@ -67816,7 +67992,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-24 10:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-25 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-25 12:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$149</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -651,23 +651,23 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(F9:F22)</f>
+        <f>SUM(F9:F24)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(G9:G22,"W")/(COUNTIF(G9:G22,"W")+COUNTIF(G9:G22,"L")),"")</f>
+        <f>IFERROR(COUNTIF(G9:G24,"W")/(COUNTIF(G9:G24,"W")+COUNTIF(G9:G24,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(G9:G22,"W")&amp;"-"&amp;COUNTIF(G9:G22,"L")</f>
+        <f>COUNTIF(G9:G24,"W")&amp;"-"&amp;COUNTIF(G9:G24,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(G9:G22,"W")+COUNTIF(G9:G22,"L")</f>
+        <f>COUNTIF(G9:G24,"W")+COUNTIF(G9:G24,"L")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTA(B9:B22)-COUNTIF(G9:G22,"W")-COUNTIF(G9:G22,"L")</f>
+        <f>COUNTA(B9:B24)-COUNTIF(G9:G24,"W")-COUNTIF(G9:G24,"L")</f>
         <v/>
       </c>
     </row>
@@ -1278,8 +1278,72 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="9" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>FLA @ CHI</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="n">
+        <v>-185</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>3.02</v>
+      </c>
+      <c r="F23" s="14">
+        <f>IF(AND(G23&lt;&gt;"W",G23&lt;&gt;"L"),"",IF(G23="W",IF(D23&gt;0,D23/100,1),IF(D23&lt;0,D23/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G23" s="11" t="inlineStr"/>
+      <c r="H23" s="10" t="inlineStr"/>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>NYI @ DAL</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="n">
+        <v>-198</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>12.71</v>
+      </c>
+      <c r="F24" s="14">
+        <f>IF(AND(G24&lt;&gt;"W",G24&lt;&gt;"L"),"",IF(G24="W",IF(D24&gt;0,D24/100,1),IF(D24&lt;0,D24/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G24" s="11" t="inlineStr"/>
+      <c r="H24" s="10" t="inlineStr"/>
+      <c r="I24" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:I22"/>
+  <autoFilter ref="A8:I24"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -1288,7 +1352,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F22">
+  <conditionalFormatting sqref="F9:F24">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -1306,7 +1370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1368,19 +1432,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H144)</f>
+        <f>SUM(H9:H149)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I144,"W")/(COUNTIF(I9:I144,"W")+COUNTIF(I9:I144,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I149,"W")/(COUNTIF(I9:I149,"W")+COUNTIF(I9:I149,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I144,"W")&amp;"-"&amp;COUNTIF(I9:I144,"L")</f>
+        <f>COUNTIF(I9:I149,"W")&amp;"-"&amp;COUNTIF(I9:I149,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I144,"W")+COUNTIF(I9:I144,"L")</f>
+        <f>COUNTIF(I9:I149,"W")+COUNTIF(I9:I149,"L")</f>
         <v/>
       </c>
     </row>
@@ -8074,8 +8138,228 @@
         </is>
       </c>
     </row>
+    <row r="145">
+      <c r="A145" s="9" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B145" s="10" t="inlineStr">
+        <is>
+          <t>FLA @ CHI</t>
+        </is>
+      </c>
+      <c r="C145" s="13" t="n">
+        <v>60.42</v>
+      </c>
+      <c r="D145" s="13" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="E145" s="13">
+        <f>IF(OR(C145="",D145=""),"",ABS(C145-D145))</f>
+        <v/>
+      </c>
+      <c r="F145" s="11" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="G145" s="12" t="n">
+        <v>-185</v>
+      </c>
+      <c r="H145" s="14">
+        <f>IF(OR(F145="",G145="",AND(I145&lt;&gt;"W",I145&lt;&gt;"L")),"",IF(I145="W",IF(G145&gt;0,G145/100,1),IF(G145&lt;0,G145/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I145" s="11" t="inlineStr"/>
+      <c r="J145" s="10" t="inlineStr"/>
+      <c r="K145" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (12:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L145" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="9" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B146" s="10" t="inlineStr">
+        <is>
+          <t>NYI @ DAL</t>
+        </is>
+      </c>
+      <c r="C146" s="13" t="n">
+        <v>68.5</v>
+      </c>
+      <c r="D146" s="13" t="n">
+        <v>81.20999999999999</v>
+      </c>
+      <c r="E146" s="13">
+        <f>IF(OR(C146="",D146=""),"",ABS(C146-D146))</f>
+        <v/>
+      </c>
+      <c r="F146" s="11" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="G146" s="12" t="n">
+        <v>-198</v>
+      </c>
+      <c r="H146" s="14">
+        <f>IF(OR(F146="",G146="",AND(I146&lt;&gt;"W",I146&lt;&gt;"L")),"",IF(I146="W",IF(G146&gt;0,G146/100,1),IF(G146&lt;0,G146/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I146" s="11" t="inlineStr"/>
+      <c r="J146" s="10" t="inlineStr"/>
+      <c r="K146" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (12:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L146" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="9" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B147" s="10" t="inlineStr">
+        <is>
+          <t>MTL @ WPG</t>
+        </is>
+      </c>
+      <c r="C147" s="13" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="D147" s="13" t="n">
+        <v>58.79</v>
+      </c>
+      <c r="E147" s="13">
+        <f>IF(OR(C147="",D147=""),"",ABS(C147-D147))</f>
+        <v/>
+      </c>
+      <c r="F147" s="11" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="G147" s="12" t="n">
+        <v>-118</v>
+      </c>
+      <c r="H147" s="14">
+        <f>IF(OR(F147="",G147="",AND(I147&lt;&gt;"W",I147&lt;&gt;"L")),"",IF(I147="W",IF(G147&gt;0,G147/100,1),IF(G147&lt;0,G147/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I147" s="11" t="inlineStr"/>
+      <c r="J147" s="10" t="inlineStr"/>
+      <c r="K147" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (12:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L147" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="9" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B148" s="10" t="inlineStr">
+        <is>
+          <t>COL @ NSH</t>
+        </is>
+      </c>
+      <c r="C148" s="13" t="n">
+        <v>68.84</v>
+      </c>
+      <c r="D148" s="13" t="n">
+        <v>58.82</v>
+      </c>
+      <c r="E148" s="13">
+        <f>IF(OR(C148="",D148=""),"",ABS(C148-D148))</f>
+        <v/>
+      </c>
+      <c r="F148" s="11" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="G148" s="12" t="n">
+        <v>-230</v>
+      </c>
+      <c r="H148" s="14">
+        <f>IF(OR(F148="",G148="",AND(I148&lt;&gt;"W",I148&lt;&gt;"L")),"",IF(I148="W",IF(G148&gt;0,G148/100,1),IF(G148&lt;0,G148/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I148" s="11" t="inlineStr"/>
+      <c r="J148" s="10" t="inlineStr"/>
+      <c r="K148" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (12:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L148" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="9" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B149" s="10" t="inlineStr">
+        <is>
+          <t>MIN @ VAN</t>
+        </is>
+      </c>
+      <c r="C149" s="13" t="n">
+        <v>90.14</v>
+      </c>
+      <c r="D149" s="13" t="n">
+        <v>46.37</v>
+      </c>
+      <c r="E149" s="13">
+        <f>IF(OR(C149="",D149=""),"",ABS(C149-D149))</f>
+        <v/>
+      </c>
+      <c r="F149" s="11" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="G149" s="12" t="n">
+        <v>-192</v>
+      </c>
+      <c r="H149" s="14">
+        <f>IF(OR(F149="",G149="",AND(I149&lt;&gt;"W",I149&lt;&gt;"L")),"",IF(I149="W",IF(G149&gt;0,G149/100,1),IF(G149&lt;0,G149/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I149" s="11" t="inlineStr"/>
+      <c r="J149" s="10" t="inlineStr"/>
+      <c r="K149" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (12:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L149" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L144"/>
+  <autoFilter ref="A8:L149"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -8084,7 +8368,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H144">
+  <conditionalFormatting sqref="H9:H149">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -67992,7 +68276,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-25 06:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-25 12:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-26 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -1302,8 +1302,16 @@
         <f>IF(AND(G23&lt;&gt;"W",G23&lt;&gt;"L"),"",IF(G23="W",IF(D23&gt;0,D23/100,1),IF(D23&lt;0,D23/100,-1)))</f>
         <v/>
       </c>
-      <c r="G23" s="11" t="inlineStr"/>
-      <c r="H23" s="10" t="inlineStr"/>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>FLA 3, CHI 2</t>
+        </is>
+      </c>
       <c r="I23" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -1334,8 +1342,16 @@
         <f>IF(AND(G24&lt;&gt;"W",G24&lt;&gt;"L"),"",IF(G24="W",IF(D24&gt;0,D24/100,1),IF(D24&lt;0,D24/100,-1)))</f>
         <v/>
       </c>
-      <c r="G24" s="11" t="inlineStr"/>
-      <c r="H24" s="10" t="inlineStr"/>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>NYI 3, DAL 6</t>
+        </is>
+      </c>
       <c r="I24" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -8169,8 +8185,16 @@
         <f>IF(OR(F145="",G145="",AND(I145&lt;&gt;"W",I145&lt;&gt;"L")),"",IF(I145="W",IF(G145&gt;0,G145/100,1),IF(G145&lt;0,G145/100,-1)))</f>
         <v/>
       </c>
-      <c r="I145" s="11" t="inlineStr"/>
-      <c r="J145" s="10" t="inlineStr"/>
+      <c r="I145" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J145" s="10" t="inlineStr">
+        <is>
+          <t>FLA 3, CHI 2</t>
+        </is>
+      </c>
       <c r="K145" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (12:00 PM CT)</t>
@@ -8213,8 +8237,16 @@
         <f>IF(OR(F146="",G146="",AND(I146&lt;&gt;"W",I146&lt;&gt;"L")),"",IF(I146="W",IF(G146&gt;0,G146/100,1),IF(G146&lt;0,G146/100,-1)))</f>
         <v/>
       </c>
-      <c r="I146" s="11" t="inlineStr"/>
-      <c r="J146" s="10" t="inlineStr"/>
+      <c r="I146" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J146" s="10" t="inlineStr">
+        <is>
+          <t>NYI 3, DAL 6</t>
+        </is>
+      </c>
       <c r="K146" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (12:00 PM CT)</t>
@@ -8257,8 +8289,16 @@
         <f>IF(OR(F147="",G147="",AND(I147&lt;&gt;"W",I147&lt;&gt;"L")),"",IF(I147="W",IF(G147&gt;0,G147/100,1),IF(G147&lt;0,G147/100,-1)))</f>
         <v/>
       </c>
-      <c r="I147" s="11" t="inlineStr"/>
-      <c r="J147" s="10" t="inlineStr"/>
+      <c r="I147" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J147" s="10" t="inlineStr">
+        <is>
+          <t>MTL 2, WPG 1</t>
+        </is>
+      </c>
       <c r="K147" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (12:00 PM CT)</t>
@@ -8301,8 +8341,16 @@
         <f>IF(OR(F148="",G148="",AND(I148&lt;&gt;"W",I148&lt;&gt;"L")),"",IF(I148="W",IF(G148&gt;0,G148/100,1),IF(G148&lt;0,G148/100,-1)))</f>
         <v/>
       </c>
-      <c r="I148" s="11" t="inlineStr"/>
-      <c r="J148" s="10" t="inlineStr"/>
+      <c r="I148" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J148" s="10" t="inlineStr">
+        <is>
+          <t>COL 2, NSH 6</t>
+        </is>
+      </c>
       <c r="K148" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (12:00 PM CT)</t>
@@ -8345,8 +8393,16 @@
         <f>IF(OR(F149="",G149="",AND(I149&lt;&gt;"W",I149&lt;&gt;"L")),"",IF(I149="W",IF(G149&gt;0,G149/100,1),IF(G149&lt;0,G149/100,-1)))</f>
         <v/>
       </c>
-      <c r="I149" s="11" t="inlineStr"/>
-      <c r="J149" s="10" t="inlineStr"/>
+      <c r="I149" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J149" s="10" t="inlineStr">
+        <is>
+          <t>MIN 4, VAN 2</t>
+        </is>
+      </c>
       <c r="K149" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (12:00 PM CT)</t>
@@ -8386,7 +8442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8599,6 +8655,38 @@
       </c>
       <c r="G8" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>50-19, +29.21 units</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>85-54, +15.52 units</t>
+        </is>
+      </c>
+      <c r="E9" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A9,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A9,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G9" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A9)</f>
         <v/>
       </c>
     </row>
@@ -68276,7 +68364,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-25 12:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-26 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-26 16:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -651,23 +651,23 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(F9:F24)</f>
+        <f>SUM(F9:F27)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(G9:G24,"W")/(COUNTIF(G9:G24,"W")+COUNTIF(G9:G24,"L")),"")</f>
+        <f>IFERROR(COUNTIF(G9:G27,"W")/(COUNTIF(G9:G27,"W")+COUNTIF(G9:G27,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(G9:G24,"W")&amp;"-"&amp;COUNTIF(G9:G24,"L")</f>
+        <f>COUNTIF(G9:G27,"W")&amp;"-"&amp;COUNTIF(G9:G27,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(G9:G24,"W")+COUNTIF(G9:G24,"L")</f>
+        <f>COUNTIF(G9:G27,"W")+COUNTIF(G9:G27,"L")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTA(B9:B24)-COUNTIF(G9:G24,"W")-COUNTIF(G9:G24,"L")</f>
+        <f>COUNTA(B9:B27)-COUNTIF(G9:G27,"W")-COUNTIF(G9:G27,"L")</f>
         <v/>
       </c>
     </row>
@@ -1358,8 +1358,104 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="9" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>LAK @ NYR</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="n">
+        <v>-135</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>12.83</v>
+      </c>
+      <c r="F25" s="14">
+        <f>IF(AND(G25&lt;&gt;"W",G25&lt;&gt;"L"),"",IF(G25="W",IF(D25&gt;0,D25/100,1),IF(D25&lt;0,D25/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G25" s="11" t="inlineStr"/>
+      <c r="H25" s="10" t="inlineStr"/>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>TOR @ CGY</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="n">
+        <v>-135</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F26" s="14">
+        <f>IF(AND(G26&lt;&gt;"W",G26&lt;&gt;"L"),"",IF(G26="W",IF(D26&gt;0,D26/100,1),IF(D26&lt;0,D26/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G26" s="11" t="inlineStr"/>
+      <c r="H26" s="10" t="inlineStr"/>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>DET @ EDM</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F27" s="14">
+        <f>IF(AND(G27&lt;&gt;"W",G27&lt;&gt;"L"),"",IF(G27="W",IF(D27&gt;0,D27/100,1),IF(D27&lt;0,D27/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G27" s="11" t="inlineStr"/>
+      <c r="H27" s="10" t="inlineStr"/>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:I24"/>
+  <autoFilter ref="A8:I27"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -1368,7 +1464,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F24">
+  <conditionalFormatting sqref="F9:F27">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -1386,7 +1482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L149"/>
+  <dimension ref="A1:L152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1448,19 +1544,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H149)</f>
+        <f>SUM(H9:H152)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I149,"W")/(COUNTIF(I9:I149,"W")+COUNTIF(I9:I149,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I152,"W")/(COUNTIF(I9:I152,"W")+COUNTIF(I9:I152,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I149,"W")&amp;"-"&amp;COUNTIF(I9:I149,"L")</f>
+        <f>COUNTIF(I9:I152,"W")&amp;"-"&amp;COUNTIF(I9:I152,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I149,"W")+COUNTIF(I9:I149,"L")</f>
+        <f>COUNTIF(I9:I152,"W")+COUNTIF(I9:I152,"L")</f>
         <v/>
       </c>
     </row>
@@ -8414,8 +8510,140 @@
         </is>
       </c>
     </row>
+    <row r="150">
+      <c r="A150" s="9" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B150" s="10" t="inlineStr">
+        <is>
+          <t>LAK @ NYR</t>
+        </is>
+      </c>
+      <c r="C150" s="13" t="n">
+        <v>58.48</v>
+      </c>
+      <c r="D150" s="13" t="n">
+        <v>71.31</v>
+      </c>
+      <c r="E150" s="13">
+        <f>IF(OR(C150="",D150=""),"",ABS(C150-D150))</f>
+        <v/>
+      </c>
+      <c r="F150" s="11" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="G150" s="12" t="n">
+        <v>-135</v>
+      </c>
+      <c r="H150" s="14">
+        <f>IF(OR(F150="",G150="",AND(I150&lt;&gt;"W",I150&lt;&gt;"L")),"",IF(I150="W",IF(G150&gt;0,G150/100,1),IF(G150&lt;0,G150/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I150" s="11" t="inlineStr"/>
+      <c r="J150" s="10" t="inlineStr"/>
+      <c r="K150" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L150" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="9" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B151" s="10" t="inlineStr">
+        <is>
+          <t>TOR @ CGY</t>
+        </is>
+      </c>
+      <c r="C151" s="13" t="n">
+        <v>83.91</v>
+      </c>
+      <c r="D151" s="13" t="n">
+        <v>73.61</v>
+      </c>
+      <c r="E151" s="13">
+        <f>IF(OR(C151="",D151=""),"",ABS(C151-D151))</f>
+        <v/>
+      </c>
+      <c r="F151" s="11" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="G151" s="12" t="n">
+        <v>-135</v>
+      </c>
+      <c r="H151" s="14">
+        <f>IF(OR(F151="",G151="",AND(I151&lt;&gt;"W",I151&lt;&gt;"L")),"",IF(I151="W",IF(G151&gt;0,G151/100,1),IF(G151&lt;0,G151/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I151" s="11" t="inlineStr"/>
+      <c r="J151" s="10" t="inlineStr"/>
+      <c r="K151" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L151" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="9" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B152" s="10" t="inlineStr">
+        <is>
+          <t>DET @ EDM</t>
+        </is>
+      </c>
+      <c r="C152" s="13" t="n">
+        <v>66.39</v>
+      </c>
+      <c r="D152" s="13" t="n">
+        <v>56.09</v>
+      </c>
+      <c r="E152" s="13">
+        <f>IF(OR(C152="",D152=""),"",ABS(C152-D152))</f>
+        <v/>
+      </c>
+      <c r="F152" s="11" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="G152" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="H152" s="14">
+        <f>IF(OR(F152="",G152="",AND(I152&lt;&gt;"W",I152&lt;&gt;"L")),"",IF(I152="W",IF(G152&gt;0,G152/100,1),IF(G152&lt;0,G152/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I152" s="11" t="inlineStr"/>
+      <c r="J152" s="10" t="inlineStr"/>
+      <c r="K152" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L152" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L149"/>
+  <autoFilter ref="A8:L152"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -8424,7 +8652,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H149">
+  <conditionalFormatting sqref="H9:H152">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -68364,7 +68592,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-26 06:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-26 16:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-27 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -1382,8 +1382,16 @@
         <f>IF(AND(G25&lt;&gt;"W",G25&lt;&gt;"L"),"",IF(G25="W",IF(D25&gt;0,D25/100,1),IF(D25&lt;0,D25/100,-1)))</f>
         <v/>
       </c>
-      <c r="G25" s="11" t="inlineStr"/>
-      <c r="H25" s="10" t="inlineStr"/>
+      <c r="G25" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>LAK 6, NYR 3</t>
+        </is>
+      </c>
       <c r="I25" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -1414,8 +1422,16 @@
         <f>IF(AND(G26&lt;&gt;"W",G26&lt;&gt;"L"),"",IF(G26="W",IF(D26&gt;0,D26/100,1),IF(D26&lt;0,D26/100,-1)))</f>
         <v/>
       </c>
-      <c r="G26" s="11" t="inlineStr"/>
-      <c r="H26" s="10" t="inlineStr"/>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>TOR 2, CGY 5</t>
+        </is>
+      </c>
       <c r="I26" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -1446,8 +1462,16 @@
         <f>IF(AND(G27&lt;&gt;"W",G27&lt;&gt;"L"),"",IF(G27="W",IF(D27&gt;0,D27/100,1),IF(D27&lt;0,D27/100,-1)))</f>
         <v/>
       </c>
-      <c r="G27" s="11" t="inlineStr"/>
-      <c r="H27" s="10" t="inlineStr"/>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>DET 4, EDM 3</t>
+        </is>
+      </c>
       <c r="I27" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -8541,8 +8565,16 @@
         <f>IF(OR(F150="",G150="",AND(I150&lt;&gt;"W",I150&lt;&gt;"L")),"",IF(I150="W",IF(G150&gt;0,G150/100,1),IF(G150&lt;0,G150/100,-1)))</f>
         <v/>
       </c>
-      <c r="I150" s="11" t="inlineStr"/>
-      <c r="J150" s="10" t="inlineStr"/>
+      <c r="I150" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J150" s="10" t="inlineStr">
+        <is>
+          <t>LAK 6, NYR 3</t>
+        </is>
+      </c>
       <c r="K150" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -8585,8 +8617,16 @@
         <f>IF(OR(F151="",G151="",AND(I151&lt;&gt;"W",I151&lt;&gt;"L")),"",IF(I151="W",IF(G151&gt;0,G151/100,1),IF(G151&lt;0,G151/100,-1)))</f>
         <v/>
       </c>
-      <c r="I151" s="11" t="inlineStr"/>
-      <c r="J151" s="10" t="inlineStr"/>
+      <c r="I151" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J151" s="10" t="inlineStr">
+        <is>
+          <t>TOR 2, CGY 5</t>
+        </is>
+      </c>
       <c r="K151" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -8629,8 +8669,16 @@
         <f>IF(OR(F152="",G152="",AND(I152&lt;&gt;"W",I152&lt;&gt;"L")),"",IF(I152="W",IF(G152&gt;0,G152/100,1),IF(G152&lt;0,G152/100,-1)))</f>
         <v/>
       </c>
-      <c r="I152" s="11" t="inlineStr"/>
-      <c r="J152" s="10" t="inlineStr"/>
+      <c r="I152" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J152" s="10" t="inlineStr">
+        <is>
+          <t>DET 4, EDM 3</t>
+        </is>
+      </c>
       <c r="K152" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -8670,7 +8718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8915,6 +8963,38 @@
       </c>
       <c r="G9" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>51-21, +28.01 units</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>86-56, +14.32 units</t>
+        </is>
+      </c>
+      <c r="E10" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A10,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A10,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G10" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A10)</f>
         <v/>
       </c>
     </row>
@@ -68592,7 +68672,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-26 16:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-27 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-27 16:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$163</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1506,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1568,19 +1568,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H152)</f>
+        <f>SUM(H9:H163)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I152,"W")/(COUNTIF(I9:I152,"W")+COUNTIF(I9:I152,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I163,"W")/(COUNTIF(I9:I163,"W")+COUNTIF(I9:I163,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I152,"W")&amp;"-"&amp;COUNTIF(I9:I152,"L")</f>
+        <f>COUNTIF(I9:I163,"W")&amp;"-"&amp;COUNTIF(I9:I163,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I152,"W")+COUNTIF(I9:I152,"L")</f>
+        <f>COUNTIF(I9:I163,"W")+COUNTIF(I9:I163,"L")</f>
         <v/>
       </c>
     </row>
@@ -8690,8 +8690,470 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B153" s="10" t="inlineStr">
+        <is>
+          <t>CBJ @ PHI</t>
+        </is>
+      </c>
+      <c r="C153" s="13" t="n">
+        <v>71.97</v>
+      </c>
+      <c r="D153" s="13" t="n">
+        <v>65.64</v>
+      </c>
+      <c r="E153" s="13">
+        <f>IF(OR(C153="",D153=""),"",ABS(C153-D153))</f>
+        <v/>
+      </c>
+      <c r="F153" s="11" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="G153" s="12" t="n"/>
+      <c r="H153" s="14">
+        <f>IF(OR(F153="",G153="",AND(I153&lt;&gt;"W",I153&lt;&gt;"L")),"",IF(I153="W",IF(G153&gt;0,G153/100,1),IF(G153&lt;0,G153/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I153" s="11" t="inlineStr"/>
+      <c r="J153" s="10" t="inlineStr"/>
+      <c r="K153" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L153" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B154" s="10" t="inlineStr">
+        <is>
+          <t>BOS @ CAR</t>
+        </is>
+      </c>
+      <c r="C154" s="13" t="n">
+        <v>83.38</v>
+      </c>
+      <c r="D154" s="13" t="n">
+        <v>90.53</v>
+      </c>
+      <c r="E154" s="13">
+        <f>IF(OR(C154="",D154=""),"",ABS(C154-D154))</f>
+        <v/>
+      </c>
+      <c r="F154" s="11" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="G154" s="12" t="n"/>
+      <c r="H154" s="14">
+        <f>IF(OR(F154="",G154="",AND(I154&lt;&gt;"W",I154&lt;&gt;"L")),"",IF(I154="W",IF(G154&gt;0,G154/100,1),IF(G154&lt;0,G154/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I154" s="11" t="inlineStr"/>
+      <c r="J154" s="10" t="inlineStr"/>
+      <c r="K154" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L154" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B155" s="10" t="inlineStr">
+        <is>
+          <t>LAK @ CHI</t>
+        </is>
+      </c>
+      <c r="C155" s="13" t="n">
+        <v>77.3</v>
+      </c>
+      <c r="D155" s="13" t="n">
+        <v>61.34</v>
+      </c>
+      <c r="E155" s="13">
+        <f>IF(OR(C155="",D155=""),"",ABS(C155-D155))</f>
+        <v/>
+      </c>
+      <c r="F155" s="11" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="G155" s="12" t="n"/>
+      <c r="H155" s="14">
+        <f>IF(OR(F155="",G155="",AND(I155&lt;&gt;"W",I155&lt;&gt;"L")),"",IF(I155="W",IF(G155&gt;0,G155/100,1),IF(G155&lt;0,G155/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I155" s="11" t="inlineStr"/>
+      <c r="J155" s="10" t="inlineStr"/>
+      <c r="K155" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L155" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B156" s="10" t="inlineStr">
+        <is>
+          <t>MTL @ STL</t>
+        </is>
+      </c>
+      <c r="C156" s="13" t="n">
+        <v>72.45999999999999</v>
+      </c>
+      <c r="D156" s="13" t="n">
+        <v>49.47</v>
+      </c>
+      <c r="E156" s="13">
+        <f>IF(OR(C156="",D156=""),"",ABS(C156-D156))</f>
+        <v/>
+      </c>
+      <c r="F156" s="11" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="G156" s="12" t="n"/>
+      <c r="H156" s="14">
+        <f>IF(OR(F156="",G156="",AND(I156&lt;&gt;"W",I156&lt;&gt;"L")),"",IF(I156="W",IF(G156&gt;0,G156/100,1),IF(G156&lt;0,G156/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I156" s="11" t="inlineStr"/>
+      <c r="J156" s="10" t="inlineStr"/>
+      <c r="K156" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L156" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B157" s="10" t="inlineStr">
+        <is>
+          <t>NYI @ NSH</t>
+        </is>
+      </c>
+      <c r="C157" s="13" t="n">
+        <v>49.58</v>
+      </c>
+      <c r="D157" s="13" t="n">
+        <v>86.8</v>
+      </c>
+      <c r="E157" s="13">
+        <f>IF(OR(C157="",D157=""),"",ABS(C157-D157))</f>
+        <v/>
+      </c>
+      <c r="F157" s="11" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="G157" s="12" t="n"/>
+      <c r="H157" s="14">
+        <f>IF(OR(F157="",G157="",AND(I157&lt;&gt;"W",I157&lt;&gt;"L")),"",IF(I157="W",IF(G157&gt;0,G157/100,1),IF(G157&lt;0,G157/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I157" s="11" t="inlineStr"/>
+      <c r="J157" s="10" t="inlineStr"/>
+      <c r="K157" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L157" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B158" s="10" t="inlineStr">
+        <is>
+          <t>NJD @ DAL</t>
+        </is>
+      </c>
+      <c r="C158" s="13" t="n">
+        <v>81.52</v>
+      </c>
+      <c r="D158" s="13" t="n">
+        <v>90.42</v>
+      </c>
+      <c r="E158" s="13">
+        <f>IF(OR(C158="",D158=""),"",ABS(C158-D158))</f>
+        <v/>
+      </c>
+      <c r="F158" s="11" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="G158" s="12" t="n"/>
+      <c r="H158" s="14">
+        <f>IF(OR(F158="",G158="",AND(I158&lt;&gt;"W",I158&lt;&gt;"L")),"",IF(I158="W",IF(G158&gt;0,G158/100,1),IF(G158&lt;0,G158/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I158" s="11" t="inlineStr"/>
+      <c r="J158" s="10" t="inlineStr"/>
+      <c r="K158" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L158" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B159" s="10" t="inlineStr">
+        <is>
+          <t>FLA @ WPG</t>
+        </is>
+      </c>
+      <c r="C159" s="13" t="n">
+        <v>78.66</v>
+      </c>
+      <c r="D159" s="13" t="n">
+        <v>67.54000000000001</v>
+      </c>
+      <c r="E159" s="13">
+        <f>IF(OR(C159="",D159=""),"",ABS(C159-D159))</f>
+        <v/>
+      </c>
+      <c r="F159" s="11" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="G159" s="12" t="n"/>
+      <c r="H159" s="14">
+        <f>IF(OR(F159="",G159="",AND(I159&lt;&gt;"W",I159&lt;&gt;"L")),"",IF(I159="W",IF(G159&gt;0,G159/100,1),IF(G159&lt;0,G159/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I159" s="11" t="inlineStr"/>
+      <c r="J159" s="10" t="inlineStr"/>
+      <c r="K159" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L159" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B160" s="10" t="inlineStr">
+        <is>
+          <t>MIN @ UTA</t>
+        </is>
+      </c>
+      <c r="C160" s="13" t="n">
+        <v>88.37</v>
+      </c>
+      <c r="D160" s="13" t="n">
+        <v>72.31</v>
+      </c>
+      <c r="E160" s="13">
+        <f>IF(OR(C160="",D160=""),"",ABS(C160-D160))</f>
+        <v/>
+      </c>
+      <c r="F160" s="11" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="G160" s="12" t="n"/>
+      <c r="H160" s="14">
+        <f>IF(OR(F160="",G160="",AND(I160&lt;&gt;"W",I160&lt;&gt;"L")),"",IF(I160="W",IF(G160&gt;0,G160/100,1),IF(G160&lt;0,G160/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I160" s="11" t="inlineStr"/>
+      <c r="J160" s="10" t="inlineStr"/>
+      <c r="K160" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L160" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B161" s="10" t="inlineStr">
+        <is>
+          <t>OTT @ VGK</t>
+        </is>
+      </c>
+      <c r="C161" s="13" t="n">
+        <v>68.69</v>
+      </c>
+      <c r="D161" s="13" t="n">
+        <v>68.03</v>
+      </c>
+      <c r="E161" s="13">
+        <f>IF(OR(C161="",D161=""),"",ABS(C161-D161))</f>
+        <v/>
+      </c>
+      <c r="F161" s="11" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="G161" s="12" t="n"/>
+      <c r="H161" s="14">
+        <f>IF(OR(F161="",G161="",AND(I161&lt;&gt;"W",I161&lt;&gt;"L")),"",IF(I161="W",IF(G161&gt;0,G161/100,1),IF(G161&lt;0,G161/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I161" s="11" t="inlineStr"/>
+      <c r="J161" s="10" t="inlineStr"/>
+      <c r="K161" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L161" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B162" s="10" t="inlineStr">
+        <is>
+          <t>VAN @ ANA</t>
+        </is>
+      </c>
+      <c r="C162" s="13" t="n">
+        <v>51.63</v>
+      </c>
+      <c r="D162" s="13" t="n">
+        <v>74.36</v>
+      </c>
+      <c r="E162" s="13">
+        <f>IF(OR(C162="",D162=""),"",ABS(C162-D162))</f>
+        <v/>
+      </c>
+      <c r="F162" s="11" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="G162" s="12" t="n"/>
+      <c r="H162" s="14">
+        <f>IF(OR(F162="",G162="",AND(I162&lt;&gt;"W",I162&lt;&gt;"L")),"",IF(I162="W",IF(G162&gt;0,G162/100,1),IF(G162&lt;0,G162/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I162" s="11" t="inlineStr"/>
+      <c r="J162" s="10" t="inlineStr"/>
+      <c r="K162" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L162" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="9" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>BUF @ SJS</t>
+        </is>
+      </c>
+      <c r="C163" s="13" t="n">
+        <v>63.39</v>
+      </c>
+      <c r="D163" s="13" t="n">
+        <v>56.62</v>
+      </c>
+      <c r="E163" s="13">
+        <f>IF(OR(C163="",D163=""),"",ABS(C163-D163))</f>
+        <v/>
+      </c>
+      <c r="F163" s="11" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="G163" s="12" t="n"/>
+      <c r="H163" s="14">
+        <f>IF(OR(F163="",G163="",AND(I163&lt;&gt;"W",I163&lt;&gt;"L")),"",IF(I163="W",IF(G163&gt;0,G163/100,1),IF(G163&lt;0,G163/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I163" s="11" t="inlineStr"/>
+      <c r="J163" s="10" t="inlineStr"/>
+      <c r="K163" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L163" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L152"/>
+  <autoFilter ref="A8:L163"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -8700,7 +9162,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H152">
+  <conditionalFormatting sqref="H9:H163">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -68672,7 +69134,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-27 06:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-27 16:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-28 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -8719,8 +8719,16 @@
         <f>IF(OR(F153="",G153="",AND(I153&lt;&gt;"W",I153&lt;&gt;"L")),"",IF(I153="W",IF(G153&gt;0,G153/100,1),IF(G153&lt;0,G153/100,-1)))</f>
         <v/>
       </c>
-      <c r="I153" s="11" t="inlineStr"/>
-      <c r="J153" s="10" t="inlineStr"/>
+      <c r="I153" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J153" s="10" t="inlineStr">
+        <is>
+          <t>CBJ 4, PHI 3</t>
+        </is>
+      </c>
       <c r="K153" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -8761,8 +8769,16 @@
         <f>IF(OR(F154="",G154="",AND(I154&lt;&gt;"W",I154&lt;&gt;"L")),"",IF(I154="W",IF(G154&gt;0,G154/100,1),IF(G154&lt;0,G154/100,-1)))</f>
         <v/>
       </c>
-      <c r="I154" s="11" t="inlineStr"/>
-      <c r="J154" s="10" t="inlineStr"/>
+      <c r="I154" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J154" s="10" t="inlineStr">
+        <is>
+          <t>BOS 1, CAR 2</t>
+        </is>
+      </c>
       <c r="K154" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -8803,8 +8819,16 @@
         <f>IF(OR(F155="",G155="",AND(I155&lt;&gt;"W",I155&lt;&gt;"L")),"",IF(I155="W",IF(G155&gt;0,G155/100,1),IF(G155&lt;0,G155/100,-1)))</f>
         <v/>
       </c>
-      <c r="I155" s="11" t="inlineStr"/>
-      <c r="J155" s="10" t="inlineStr"/>
+      <c r="I155" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J155" s="10" t="inlineStr">
+        <is>
+          <t>LAK 1, CHI 2</t>
+        </is>
+      </c>
       <c r="K155" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -8845,8 +8869,16 @@
         <f>IF(OR(F156="",G156="",AND(I156&lt;&gt;"W",I156&lt;&gt;"L")),"",IF(I156="W",IF(G156&gt;0,G156/100,1),IF(G156&lt;0,G156/100,-1)))</f>
         <v/>
       </c>
-      <c r="I156" s="11" t="inlineStr"/>
-      <c r="J156" s="10" t="inlineStr"/>
+      <c r="I156" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J156" s="10" t="inlineStr">
+        <is>
+          <t>MTL 2, STL 0</t>
+        </is>
+      </c>
       <c r="K156" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -8887,8 +8919,16 @@
         <f>IF(OR(F157="",G157="",AND(I157&lt;&gt;"W",I157&lt;&gt;"L")),"",IF(I157="W",IF(G157&gt;0,G157/100,1),IF(G157&lt;0,G157/100,-1)))</f>
         <v/>
       </c>
-      <c r="I157" s="11" t="inlineStr"/>
-      <c r="J157" s="10" t="inlineStr"/>
+      <c r="I157" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J157" s="10" t="inlineStr">
+        <is>
+          <t>NYI 4, NSH 3</t>
+        </is>
+      </c>
       <c r="K157" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -8929,8 +8969,16 @@
         <f>IF(OR(F158="",G158="",AND(I158&lt;&gt;"W",I158&lt;&gt;"L")),"",IF(I158="W",IF(G158&gt;0,G158/100,1),IF(G158&lt;0,G158/100,-1)))</f>
         <v/>
       </c>
-      <c r="I158" s="11" t="inlineStr"/>
-      <c r="J158" s="10" t="inlineStr"/>
+      <c r="I158" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J158" s="10" t="inlineStr">
+        <is>
+          <t>NJD 5, DAL 1</t>
+        </is>
+      </c>
       <c r="K158" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -8971,8 +9019,16 @@
         <f>IF(OR(F159="",G159="",AND(I159&lt;&gt;"W",I159&lt;&gt;"L")),"",IF(I159="W",IF(G159&gt;0,G159/100,1),IF(G159&lt;0,G159/100,-1)))</f>
         <v/>
       </c>
-      <c r="I159" s="11" t="inlineStr"/>
-      <c r="J159" s="10" t="inlineStr"/>
+      <c r="I159" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J159" s="10" t="inlineStr">
+        <is>
+          <t>FLA 5, WPG 1</t>
+        </is>
+      </c>
       <c r="K159" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -9013,8 +9069,16 @@
         <f>IF(OR(F160="",G160="",AND(I160&lt;&gt;"W",I160&lt;&gt;"L")),"",IF(I160="W",IF(G160&gt;0,G160/100,1),IF(G160&lt;0,G160/100,-1)))</f>
         <v/>
       </c>
-      <c r="I160" s="11" t="inlineStr"/>
-      <c r="J160" s="10" t="inlineStr"/>
+      <c r="I160" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J160" s="10" t="inlineStr">
+        <is>
+          <t>MIN 3, UTA 1</t>
+        </is>
+      </c>
       <c r="K160" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -9055,8 +9119,16 @@
         <f>IF(OR(F161="",G161="",AND(I161&lt;&gt;"W",I161&lt;&gt;"L")),"",IF(I161="W",IF(G161&gt;0,G161/100,1),IF(G161&lt;0,G161/100,-1)))</f>
         <v/>
       </c>
-      <c r="I161" s="11" t="inlineStr"/>
-      <c r="J161" s="10" t="inlineStr"/>
+      <c r="I161" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J161" s="10" t="inlineStr">
+        <is>
+          <t>OTT 1, VGK 4</t>
+        </is>
+      </c>
       <c r="K161" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -9097,8 +9169,16 @@
         <f>IF(OR(F162="",G162="",AND(I162&lt;&gt;"W",I162&lt;&gt;"L")),"",IF(I162="W",IF(G162&gt;0,G162/100,1),IF(G162&lt;0,G162/100,-1)))</f>
         <v/>
       </c>
-      <c r="I162" s="11" t="inlineStr"/>
-      <c r="J162" s="10" t="inlineStr"/>
+      <c r="I162" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J162" s="10" t="inlineStr">
+        <is>
+          <t>VAN 6, ANA 5</t>
+        </is>
+      </c>
       <c r="K162" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -9139,8 +9219,16 @@
         <f>IF(OR(F163="",G163="",AND(I163&lt;&gt;"W",I163&lt;&gt;"L")),"",IF(I163="W",IF(G163&gt;0,G163/100,1),IF(G163&lt;0,G163/100,-1)))</f>
         <v/>
       </c>
-      <c r="I163" s="11" t="inlineStr"/>
-      <c r="J163" s="10" t="inlineStr"/>
+      <c r="I163" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J163" s="10" t="inlineStr">
+        <is>
+          <t>BUF 2, SJS 0</t>
+        </is>
+      </c>
       <c r="K163" s="10" t="inlineStr">
         <is>
           <t>no line at pick time</t>
@@ -9180,7 +9268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9457,6 +9545,38 @@
       </c>
       <c r="G10" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>51-21, +28.01 units</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>86-56, +14.32 units</t>
+        </is>
+      </c>
+      <c r="E11" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A11,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A11,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G11" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A11)</f>
         <v/>
       </c>
     </row>
@@ -69134,7 +69254,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-27 16:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-28 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-28 16:30 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$163</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$167</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -651,23 +651,23 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(F9:F27)</f>
+        <f>SUM(F9:F29)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(G9:G27,"W")/(COUNTIF(G9:G27,"W")+COUNTIF(G9:G27,"L")),"")</f>
+        <f>IFERROR(COUNTIF(G9:G29,"W")/(COUNTIF(G9:G29,"W")+COUNTIF(G9:G29,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(G9:G27,"W")&amp;"-"&amp;COUNTIF(G9:G27,"L")</f>
+        <f>COUNTIF(G9:G29,"W")&amp;"-"&amp;COUNTIF(G9:G29,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(G9:G27,"W")+COUNTIF(G9:G27,"L")</f>
+        <f>COUNTIF(G9:G29,"W")+COUNTIF(G9:G29,"L")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTA(B9:B27)-COUNTIF(G9:G27,"W")-COUNTIF(G9:G27,"L")</f>
+        <f>COUNTA(B9:B29)-COUNTIF(G9:G29,"W")-COUNTIF(G9:G29,"L")</f>
         <v/>
       </c>
     </row>
@@ -1478,8 +1478,72 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="9" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>CGY @ EDM</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>11.66</v>
+      </c>
+      <c r="F28" s="14">
+        <f>IF(AND(G28&lt;&gt;"W",G28&lt;&gt;"L"),"",IF(G28="W",IF(D28&gt;0,D28/100,1),IF(D28&lt;0,D28/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G28" s="11" t="inlineStr"/>
+      <c r="H28" s="10" t="inlineStr"/>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>TOR @ SEA</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="n">
+        <v>-135</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="F29" s="14">
+        <f>IF(AND(G29&lt;&gt;"W",G29&lt;&gt;"L"),"",IF(G29="W",IF(D29&gt;0,D29/100,1),IF(D29&lt;0,D29/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G29" s="11" t="inlineStr"/>
+      <c r="H29" s="10" t="inlineStr"/>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:I27"/>
+  <autoFilter ref="A8:I29"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -1488,7 +1552,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F27">
+  <conditionalFormatting sqref="F9:F29">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -1506,7 +1570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L163"/>
+  <dimension ref="A1:L167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1568,19 +1632,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H163)</f>
+        <f>SUM(H9:H167)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I163,"W")/(COUNTIF(I9:I163,"W")+COUNTIF(I9:I163,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I167,"W")/(COUNTIF(I9:I167,"W")+COUNTIF(I9:I167,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I163,"W")&amp;"-"&amp;COUNTIF(I9:I163,"L")</f>
+        <f>COUNTIF(I9:I167,"W")&amp;"-"&amp;COUNTIF(I9:I167,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I163,"W")+COUNTIF(I9:I163,"L")</f>
+        <f>COUNTIF(I9:I167,"W")+COUNTIF(I9:I167,"L")</f>
         <v/>
       </c>
     </row>
@@ -9240,8 +9304,184 @@
         </is>
       </c>
     </row>
+    <row r="164">
+      <c r="A164" s="9" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B164" s="10" t="inlineStr">
+        <is>
+          <t>PHI @ WSH</t>
+        </is>
+      </c>
+      <c r="C164" s="13" t="n">
+        <v>75.98999999999999</v>
+      </c>
+      <c r="D164" s="13" t="n">
+        <v>76.61</v>
+      </c>
+      <c r="E164" s="13">
+        <f>IF(OR(C164="",D164=""),"",ABS(C164-D164))</f>
+        <v/>
+      </c>
+      <c r="F164" s="11" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="G164" s="12" t="n">
+        <v>-245</v>
+      </c>
+      <c r="H164" s="14">
+        <f>IF(OR(F164="",G164="",AND(I164&lt;&gt;"W",I164&lt;&gt;"L")),"",IF(I164="W",IF(G164&gt;0,G164/100,1),IF(G164&lt;0,G164/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I164" s="11" t="inlineStr"/>
+      <c r="J164" s="10" t="inlineStr"/>
+      <c r="K164" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:30 PM CT)</t>
+        </is>
+      </c>
+      <c r="L164" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="9" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B165" s="10" t="inlineStr">
+        <is>
+          <t>CGY @ EDM</t>
+        </is>
+      </c>
+      <c r="C165" s="13" t="n">
+        <v>82.02</v>
+      </c>
+      <c r="D165" s="13" t="n">
+        <v>70.36</v>
+      </c>
+      <c r="E165" s="13">
+        <f>IF(OR(C165="",D165=""),"",ABS(C165-D165))</f>
+        <v/>
+      </c>
+      <c r="F165" s="11" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="G165" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="H165" s="14">
+        <f>IF(OR(F165="",G165="",AND(I165&lt;&gt;"W",I165&lt;&gt;"L")),"",IF(I165="W",IF(G165&gt;0,G165/100,1),IF(G165&lt;0,G165/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I165" s="11" t="inlineStr"/>
+      <c r="J165" s="10" t="inlineStr"/>
+      <c r="K165" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:30 PM CT)</t>
+        </is>
+      </c>
+      <c r="L165" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="9" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B166" s="10" t="inlineStr">
+        <is>
+          <t>NJD @ COL</t>
+        </is>
+      </c>
+      <c r="C166" s="13" t="n">
+        <v>87.98</v>
+      </c>
+      <c r="D166" s="13" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="E166" s="13">
+        <f>IF(OR(C166="",D166=""),"",ABS(C166-D166))</f>
+        <v/>
+      </c>
+      <c r="F166" s="11" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="G166" s="12" t="n">
+        <v>124</v>
+      </c>
+      <c r="H166" s="14">
+        <f>IF(OR(F166="",G166="",AND(I166&lt;&gt;"W",I166&lt;&gt;"L")),"",IF(I166="W",IF(G166&gt;0,G166/100,1),IF(G166&lt;0,G166/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I166" s="11" t="inlineStr"/>
+      <c r="J166" s="10" t="inlineStr"/>
+      <c r="K166" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:30 PM CT)</t>
+        </is>
+      </c>
+      <c r="L166" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="9" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B167" s="10" t="inlineStr">
+        <is>
+          <t>TOR @ SEA</t>
+        </is>
+      </c>
+      <c r="C167" s="13" t="n">
+        <v>57.98</v>
+      </c>
+      <c r="D167" s="13" t="n">
+        <v>49.86</v>
+      </c>
+      <c r="E167" s="13">
+        <f>IF(OR(C167="",D167=""),"",ABS(C167-D167))</f>
+        <v/>
+      </c>
+      <c r="F167" s="11" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="G167" s="12" t="n">
+        <v>-135</v>
+      </c>
+      <c r="H167" s="14">
+        <f>IF(OR(F167="",G167="",AND(I167&lt;&gt;"W",I167&lt;&gt;"L")),"",IF(I167="W",IF(G167&gt;0,G167/100,1),IF(G167&lt;0,G167/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I167" s="11" t="inlineStr"/>
+      <c r="J167" s="10" t="inlineStr"/>
+      <c r="K167" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:30 PM CT)</t>
+        </is>
+      </c>
+      <c r="L167" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L163"/>
+  <autoFilter ref="A8:L167"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -9250,7 +9490,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H163">
+  <conditionalFormatting sqref="H9:H167">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -69254,7 +69494,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-28 06:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-28 16:30 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-29 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -1502,8 +1502,16 @@
         <f>IF(AND(G28&lt;&gt;"W",G28&lt;&gt;"L"),"",IF(G28="W",IF(D28&gt;0,D28/100,1),IF(D28&lt;0,D28/100,-1)))</f>
         <v/>
       </c>
-      <c r="G28" s="11" t="inlineStr"/>
-      <c r="H28" s="10" t="inlineStr"/>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>CGY 0, EDM 4</t>
+        </is>
+      </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -1534,8 +1542,16 @@
         <f>IF(AND(G29&lt;&gt;"W",G29&lt;&gt;"L"),"",IF(G29="W",IF(D29&gt;0,D29/100,1),IF(D29&lt;0,D29/100,-1)))</f>
         <v/>
       </c>
-      <c r="G29" s="11" t="inlineStr"/>
-      <c r="H29" s="10" t="inlineStr"/>
+      <c r="G29" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>TOR 4, SEA 5</t>
+        </is>
+      </c>
       <c r="I29" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -9335,8 +9351,16 @@
         <f>IF(OR(F164="",G164="",AND(I164&lt;&gt;"W",I164&lt;&gt;"L")),"",IF(I164="W",IF(G164&gt;0,G164/100,1),IF(G164&lt;0,G164/100,-1)))</f>
         <v/>
       </c>
-      <c r="I164" s="11" t="inlineStr"/>
-      <c r="J164" s="10" t="inlineStr"/>
+      <c r="I164" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J164" s="10" t="inlineStr">
+        <is>
+          <t>PHI 2, WSH 5</t>
+        </is>
+      </c>
       <c r="K164" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:30 PM CT)</t>
@@ -9379,8 +9403,16 @@
         <f>IF(OR(F165="",G165="",AND(I165&lt;&gt;"W",I165&lt;&gt;"L")),"",IF(I165="W",IF(G165&gt;0,G165/100,1),IF(G165&lt;0,G165/100,-1)))</f>
         <v/>
       </c>
-      <c r="I165" s="11" t="inlineStr"/>
-      <c r="J165" s="10" t="inlineStr"/>
+      <c r="I165" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J165" s="10" t="inlineStr">
+        <is>
+          <t>CGY 0, EDM 4</t>
+        </is>
+      </c>
       <c r="K165" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:30 PM CT)</t>
@@ -9423,8 +9455,16 @@
         <f>IF(OR(F166="",G166="",AND(I166&lt;&gt;"W",I166&lt;&gt;"L")),"",IF(I166="W",IF(G166&gt;0,G166/100,1),IF(G166&lt;0,G166/100,-1)))</f>
         <v/>
       </c>
-      <c r="I166" s="11" t="inlineStr"/>
-      <c r="J166" s="10" t="inlineStr"/>
+      <c r="I166" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J166" s="10" t="inlineStr">
+        <is>
+          <t>NJD 2, COL 5</t>
+        </is>
+      </c>
       <c r="K166" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:30 PM CT)</t>
@@ -9467,8 +9507,16 @@
         <f>IF(OR(F167="",G167="",AND(I167&lt;&gt;"W",I167&lt;&gt;"L")),"",IF(I167="W",IF(G167&gt;0,G167/100,1),IF(G167&lt;0,G167/100,-1)))</f>
         <v/>
       </c>
-      <c r="I167" s="11" t="inlineStr"/>
-      <c r="J167" s="10" t="inlineStr"/>
+      <c r="I167" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J167" s="10" t="inlineStr">
+        <is>
+          <t>TOR 4, SEA 5</t>
+        </is>
+      </c>
       <c r="K167" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:30 PM CT)</t>
@@ -9508,7 +9556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9817,6 +9865,38 @@
       </c>
       <c r="G11" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>51-23, +25.66 units</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>87-59, +11.97 units</t>
+        </is>
+      </c>
+      <c r="E12" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A12,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A12,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G12" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A12)</f>
         <v/>
       </c>
     </row>
@@ -69494,7 +69574,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-28 16:30 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-29 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-29 16:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$167</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$178</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -651,23 +651,23 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(F9:F29)</f>
+        <f>SUM(F9:F33)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(G9:G29,"W")/(COUNTIF(G9:G29,"W")+COUNTIF(G9:G29,"L")),"")</f>
+        <f>IFERROR(COUNTIF(G9:G33,"W")/(COUNTIF(G9:G33,"W")+COUNTIF(G9:G33,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(G9:G29,"W")&amp;"-"&amp;COUNTIF(G9:G29,"L")</f>
+        <f>COUNTIF(G9:G33,"W")&amp;"-"&amp;COUNTIF(G9:G33,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(G9:G29,"W")+COUNTIF(G9:G29,"L")</f>
+        <f>COUNTIF(G9:G33,"W")+COUNTIF(G9:G33,"L")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTA(B9:B29)-COUNTIF(G9:G29,"W")-COUNTIF(G9:G29,"L")</f>
+        <f>COUNTA(B9:B33)-COUNTIF(G9:G33,"W")-COUNTIF(G9:G33,"L")</f>
         <v/>
       </c>
     </row>
@@ -1558,8 +1558,136 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>CHI @ DET</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="n">
+        <v>136</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>6.05</v>
+      </c>
+      <c r="F30" s="14">
+        <f>IF(AND(G30&lt;&gt;"W",G30&lt;&gt;"L"),"",IF(G30="W",IF(D30&gt;0,D30/100,1),IF(D30&lt;0,D30/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G30" s="11" t="inlineStr"/>
+      <c r="H30" s="10" t="inlineStr"/>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>WSH @ NSH</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="n">
+        <v>-112</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <v>13.21</v>
+      </c>
+      <c r="F31" s="14">
+        <f>IF(AND(G31&lt;&gt;"W",G31&lt;&gt;"L"),"",IF(G31="W",IF(D31&gt;0,D31/100,1),IF(D31&lt;0,D31/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G31" s="11" t="inlineStr"/>
+      <c r="H31" s="10" t="inlineStr"/>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>NYI @ MIN</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="n">
+        <v>-192</v>
+      </c>
+      <c r="E32" s="13" t="n">
+        <v>4.87</v>
+      </c>
+      <c r="F32" s="14">
+        <f>IF(AND(G32&lt;&gt;"W",G32&lt;&gt;"L"),"",IF(G32="W",IF(D32&gt;0,D32/100,1),IF(D32&lt;0,D32/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G32" s="11" t="inlineStr"/>
+      <c r="H32" s="10" t="inlineStr"/>
+      <c r="I32" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>OTT @ LAK</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="n">
+        <v>-125</v>
+      </c>
+      <c r="E33" s="13" t="n">
+        <v>2.53</v>
+      </c>
+      <c r="F33" s="14">
+        <f>IF(AND(G33&lt;&gt;"W",G33&lt;&gt;"L"),"",IF(G33="W",IF(D33&gt;0,D33/100,1),IF(D33&lt;0,D33/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G33" s="11" t="inlineStr"/>
+      <c r="H33" s="10" t="inlineStr"/>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:I29"/>
+  <autoFilter ref="A8:I33"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -1568,7 +1696,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F29">
+  <conditionalFormatting sqref="F9:F33">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -1586,7 +1714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L167"/>
+  <dimension ref="A1:L178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1648,19 +1776,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H167)</f>
+        <f>SUM(H9:H178)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I167,"W")/(COUNTIF(I9:I167,"W")+COUNTIF(I9:I167,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I178,"W")/(COUNTIF(I9:I178,"W")+COUNTIF(I9:I178,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I167,"W")&amp;"-"&amp;COUNTIF(I9:I167,"L")</f>
+        <f>COUNTIF(I9:I178,"W")&amp;"-"&amp;COUNTIF(I9:I178,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I167,"W")+COUNTIF(I9:I167,"L")</f>
+        <f>COUNTIF(I9:I178,"W")+COUNTIF(I9:I178,"L")</f>
         <v/>
       </c>
     </row>
@@ -9528,8 +9656,492 @@
         </is>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B168" s="10" t="inlineStr">
+        <is>
+          <t>WPG @ TBL</t>
+        </is>
+      </c>
+      <c r="C168" s="13" t="n">
+        <v>59.07</v>
+      </c>
+      <c r="D168" s="13" t="n">
+        <v>67.69</v>
+      </c>
+      <c r="E168" s="13">
+        <f>IF(OR(C168="",D168=""),"",ABS(C168-D168))</f>
+        <v/>
+      </c>
+      <c r="F168" s="11" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="G168" s="12" t="n">
+        <v>-218</v>
+      </c>
+      <c r="H168" s="14">
+        <f>IF(OR(F168="",G168="",AND(I168&lt;&gt;"W",I168&lt;&gt;"L")),"",IF(I168="W",IF(G168&gt;0,G168/100,1),IF(G168&lt;0,G168/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I168" s="11" t="inlineStr"/>
+      <c r="J168" s="10" t="inlineStr"/>
+      <c r="K168" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L168" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B169" s="10" t="inlineStr">
+        <is>
+          <t>UTA @ PIT</t>
+        </is>
+      </c>
+      <c r="C169" s="13" t="n">
+        <v>62.85</v>
+      </c>
+      <c r="D169" s="13" t="n">
+        <v>81.18000000000001</v>
+      </c>
+      <c r="E169" s="13">
+        <f>IF(OR(C169="",D169=""),"",ABS(C169-D169))</f>
+        <v/>
+      </c>
+      <c r="F169" s="11" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="G169" s="12" t="n">
+        <v>114</v>
+      </c>
+      <c r="H169" s="14">
+        <f>IF(OR(F169="",G169="",AND(I169&lt;&gt;"W",I169&lt;&gt;"L")),"",IF(I169="W",IF(G169&gt;0,G169/100,1),IF(G169&lt;0,G169/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I169" s="11" t="inlineStr"/>
+      <c r="J169" s="10" t="inlineStr"/>
+      <c r="K169" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L169" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B170" s="10" t="inlineStr">
+        <is>
+          <t>CBJ @ CAR</t>
+        </is>
+      </c>
+      <c r="C170" s="13" t="n">
+        <v>64.01000000000001</v>
+      </c>
+      <c r="D170" s="13" t="n">
+        <v>84.23999999999999</v>
+      </c>
+      <c r="E170" s="13">
+        <f>IF(OR(C170="",D170=""),"",ABS(C170-D170))</f>
+        <v/>
+      </c>
+      <c r="F170" s="11" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="G170" s="12" t="n">
+        <v>-258</v>
+      </c>
+      <c r="H170" s="14">
+        <f>IF(OR(F170="",G170="",AND(I170&lt;&gt;"W",I170&lt;&gt;"L")),"",IF(I170="W",IF(G170&gt;0,G170/100,1),IF(G170&lt;0,G170/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I170" s="11" t="inlineStr"/>
+      <c r="J170" s="10" t="inlineStr"/>
+      <c r="K170" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L170" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B171" s="10" t="inlineStr">
+        <is>
+          <t>CHI @ DET</t>
+        </is>
+      </c>
+      <c r="C171" s="13" t="n">
+        <v>75.69</v>
+      </c>
+      <c r="D171" s="13" t="n">
+        <v>69.64</v>
+      </c>
+      <c r="E171" s="13">
+        <f>IF(OR(C171="",D171=""),"",ABS(C171-D171))</f>
+        <v/>
+      </c>
+      <c r="F171" s="11" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="G171" s="12" t="n">
+        <v>136</v>
+      </c>
+      <c r="H171" s="14">
+        <f>IF(OR(F171="",G171="",AND(I171&lt;&gt;"W",I171&lt;&gt;"L")),"",IF(I171="W",IF(G171&gt;0,G171/100,1),IF(G171&lt;0,G171/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I171" s="11" t="inlineStr"/>
+      <c r="J171" s="10" t="inlineStr"/>
+      <c r="K171" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L171" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B172" s="10" t="inlineStr">
+        <is>
+          <t>BOS @ STL</t>
+        </is>
+      </c>
+      <c r="C172" s="13" t="n">
+        <v>55.76</v>
+      </c>
+      <c r="D172" s="13" t="n">
+        <v>72.7</v>
+      </c>
+      <c r="E172" s="13">
+        <f>IF(OR(C172="",D172=""),"",ABS(C172-D172))</f>
+        <v/>
+      </c>
+      <c r="F172" s="11" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="G172" s="12" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H172" s="14">
+        <f>IF(OR(F172="",G172="",AND(I172&lt;&gt;"W",I172&lt;&gt;"L")),"",IF(I172="W",IF(G172&gt;0,G172/100,1),IF(G172&lt;0,G172/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I172" s="11" t="inlineStr"/>
+      <c r="J172" s="10" t="inlineStr"/>
+      <c r="K172" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L172" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B173" s="10" t="inlineStr">
+        <is>
+          <t>WSH @ NSH</t>
+        </is>
+      </c>
+      <c r="C173" s="13" t="n">
+        <v>80.93000000000001</v>
+      </c>
+      <c r="D173" s="13" t="n">
+        <v>67.72</v>
+      </c>
+      <c r="E173" s="13">
+        <f>IF(OR(C173="",D173=""),"",ABS(C173-D173))</f>
+        <v/>
+      </c>
+      <c r="F173" s="11" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="G173" s="12" t="n">
+        <v>-112</v>
+      </c>
+      <c r="H173" s="14">
+        <f>IF(OR(F173="",G173="",AND(I173&lt;&gt;"W",I173&lt;&gt;"L")),"",IF(I173="W",IF(G173&gt;0,G173/100,1),IF(G173&lt;0,G173/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I173" s="11" t="inlineStr"/>
+      <c r="J173" s="10" t="inlineStr"/>
+      <c r="K173" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L173" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B174" s="10" t="inlineStr">
+        <is>
+          <t>MTL @ DAL</t>
+        </is>
+      </c>
+      <c r="C174" s="13" t="n">
+        <v>67.3</v>
+      </c>
+      <c r="D174" s="13" t="n">
+        <v>52.02</v>
+      </c>
+      <c r="E174" s="13">
+        <f>IF(OR(C174="",D174=""),"",ABS(C174-D174))</f>
+        <v/>
+      </c>
+      <c r="F174" s="11" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="G174" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="H174" s="14">
+        <f>IF(OR(F174="",G174="",AND(I174&lt;&gt;"W",I174&lt;&gt;"L")),"",IF(I174="W",IF(G174&gt;0,G174/100,1),IF(G174&lt;0,G174/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I174" s="11" t="inlineStr"/>
+      <c r="J174" s="10" t="inlineStr"/>
+      <c r="K174" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L174" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B175" s="10" t="inlineStr">
+        <is>
+          <t>NYI @ MIN</t>
+        </is>
+      </c>
+      <c r="C175" s="13" t="n">
+        <v>72.28</v>
+      </c>
+      <c r="D175" s="13" t="n">
+        <v>77.15000000000001</v>
+      </c>
+      <c r="E175" s="13">
+        <f>IF(OR(C175="",D175=""),"",ABS(C175-D175))</f>
+        <v/>
+      </c>
+      <c r="F175" s="11" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="G175" s="12" t="n">
+        <v>-192</v>
+      </c>
+      <c r="H175" s="14">
+        <f>IF(OR(F175="",G175="",AND(I175&lt;&gt;"W",I175&lt;&gt;"L")),"",IF(I175="W",IF(G175&gt;0,G175/100,1),IF(G175&lt;0,G175/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I175" s="11" t="inlineStr"/>
+      <c r="J175" s="10" t="inlineStr"/>
+      <c r="K175" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L175" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B176" s="10" t="inlineStr">
+        <is>
+          <t>BUF @ ANA</t>
+        </is>
+      </c>
+      <c r="C176" s="13" t="n">
+        <v>79.29000000000001</v>
+      </c>
+      <c r="D176" s="13" t="n">
+        <v>63.17</v>
+      </c>
+      <c r="E176" s="13">
+        <f>IF(OR(C176="",D176=""),"",ABS(C176-D176))</f>
+        <v/>
+      </c>
+      <c r="F176" s="11" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="G176" s="12" t="n">
+        <v>-142</v>
+      </c>
+      <c r="H176" s="14">
+        <f>IF(OR(F176="",G176="",AND(I176&lt;&gt;"W",I176&lt;&gt;"L")),"",IF(I176="W",IF(G176&gt;0,G176/100,1),IF(G176&lt;0,G176/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I176" s="11" t="inlineStr"/>
+      <c r="J176" s="10" t="inlineStr"/>
+      <c r="K176" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L176" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B177" s="10" t="inlineStr">
+        <is>
+          <t>OTT @ LAK</t>
+        </is>
+      </c>
+      <c r="C177" s="13" t="n">
+        <v>66.84</v>
+      </c>
+      <c r="D177" s="13" t="n">
+        <v>64.31</v>
+      </c>
+      <c r="E177" s="13">
+        <f>IF(OR(C177="",D177=""),"",ABS(C177-D177))</f>
+        <v/>
+      </c>
+      <c r="F177" s="11" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="G177" s="12" t="n">
+        <v>-125</v>
+      </c>
+      <c r="H177" s="14">
+        <f>IF(OR(F177="",G177="",AND(I177&lt;&gt;"W",I177&lt;&gt;"L")),"",IF(I177="W",IF(G177&gt;0,G177/100,1),IF(G177&lt;0,G177/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I177" s="11" t="inlineStr"/>
+      <c r="J177" s="10" t="inlineStr"/>
+      <c r="K177" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L177" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="9" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B178" s="10" t="inlineStr">
+        <is>
+          <t>VAN @ SJS</t>
+        </is>
+      </c>
+      <c r="C178" s="13" t="n">
+        <v>76.83</v>
+      </c>
+      <c r="D178" s="13" t="n">
+        <v>60.71</v>
+      </c>
+      <c r="E178" s="13">
+        <f>IF(OR(C178="",D178=""),"",ABS(C178-D178))</f>
+        <v/>
+      </c>
+      <c r="F178" s="11" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="G178" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="H178" s="14">
+        <f>IF(OR(F178="",G178="",AND(I178&lt;&gt;"W",I178&lt;&gt;"L")),"",IF(I178="W",IF(G178&gt;0,G178/100,1),IF(G178&lt;0,G178/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I178" s="11" t="inlineStr"/>
+      <c r="J178" s="10" t="inlineStr"/>
+      <c r="K178" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (4:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L178" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L167"/>
+  <autoFilter ref="A8:L178"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -9538,7 +10150,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H167">
+  <conditionalFormatting sqref="H9:H178">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -69574,7 +70186,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-29 06:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-29 16:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-30 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -1582,8 +1582,16 @@
         <f>IF(AND(G30&lt;&gt;"W",G30&lt;&gt;"L"),"",IF(G30="W",IF(D30&gt;0,D30/100,1),IF(D30&lt;0,D30/100,-1)))</f>
         <v/>
       </c>
-      <c r="G30" s="11" t="inlineStr"/>
-      <c r="H30" s="10" t="inlineStr"/>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>CHI 1, DET 4</t>
+        </is>
+      </c>
       <c r="I30" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -1614,8 +1622,16 @@
         <f>IF(AND(G31&lt;&gt;"W",G31&lt;&gt;"L"),"",IF(G31="W",IF(D31&gt;0,D31/100,1),IF(D31&lt;0,D31/100,-1)))</f>
         <v/>
       </c>
-      <c r="G31" s="11" t="inlineStr"/>
-      <c r="H31" s="10" t="inlineStr"/>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>WSH 4, NSH 3</t>
+        </is>
+      </c>
       <c r="I31" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -1646,8 +1662,16 @@
         <f>IF(AND(G32&lt;&gt;"W",G32&lt;&gt;"L"),"",IF(G32="W",IF(D32&gt;0,D32/100,1),IF(D32&lt;0,D32/100,-1)))</f>
         <v/>
       </c>
-      <c r="G32" s="11" t="inlineStr"/>
-      <c r="H32" s="10" t="inlineStr"/>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H32" s="10" t="inlineStr">
+        <is>
+          <t>NYI 4, MIN 3</t>
+        </is>
+      </c>
       <c r="I32" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -1678,8 +1702,16 @@
         <f>IF(AND(G33&lt;&gt;"W",G33&lt;&gt;"L"),"",IF(G33="W",IF(D33&gt;0,D33/100,1),IF(D33&lt;0,D33/100,-1)))</f>
         <v/>
       </c>
-      <c r="G33" s="11" t="inlineStr"/>
-      <c r="H33" s="10" t="inlineStr"/>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>OTT 5, LAK 6</t>
+        </is>
+      </c>
       <c r="I33" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
@@ -1748,7 +1780,7 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Today's rule: Bet the pick when it has a line from -198 to +150 and a differential of 14.61 or less; home or away.</t>
+          <t>Today's rule: Bet the pick when it has any line up to +136 and a differential of 31.34 or less; home picks only.</t>
         </is>
       </c>
     </row>
@@ -9687,8 +9719,16 @@
         <f>IF(OR(F168="",G168="",AND(I168&lt;&gt;"W",I168&lt;&gt;"L")),"",IF(I168="W",IF(G168&gt;0,G168/100,1),IF(G168&lt;0,G168/100,-1)))</f>
         <v/>
       </c>
-      <c r="I168" s="11" t="inlineStr"/>
-      <c r="J168" s="10" t="inlineStr"/>
+      <c r="I168" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J168" s="10" t="inlineStr">
+        <is>
+          <t>WPG 4, TBL 6</t>
+        </is>
+      </c>
       <c r="K168" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -9731,8 +9771,16 @@
         <f>IF(OR(F169="",G169="",AND(I169&lt;&gt;"W",I169&lt;&gt;"L")),"",IF(I169="W",IF(G169&gt;0,G169/100,1),IF(G169&lt;0,G169/100,-1)))</f>
         <v/>
       </c>
-      <c r="I169" s="11" t="inlineStr"/>
-      <c r="J169" s="10" t="inlineStr"/>
+      <c r="I169" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J169" s="10" t="inlineStr">
+        <is>
+          <t>UTA 4, PIT 3</t>
+        </is>
+      </c>
       <c r="K169" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -9775,8 +9823,16 @@
         <f>IF(OR(F170="",G170="",AND(I170&lt;&gt;"W",I170&lt;&gt;"L")),"",IF(I170="W",IF(G170&gt;0,G170/100,1),IF(G170&lt;0,G170/100,-1)))</f>
         <v/>
       </c>
-      <c r="I170" s="11" t="inlineStr"/>
-      <c r="J170" s="10" t="inlineStr"/>
+      <c r="I170" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J170" s="10" t="inlineStr">
+        <is>
+          <t>CBJ 2, CAR 3</t>
+        </is>
+      </c>
       <c r="K170" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -9819,8 +9875,16 @@
         <f>IF(OR(F171="",G171="",AND(I171&lt;&gt;"W",I171&lt;&gt;"L")),"",IF(I171="W",IF(G171&gt;0,G171/100,1),IF(G171&lt;0,G171/100,-1)))</f>
         <v/>
       </c>
-      <c r="I171" s="11" t="inlineStr"/>
-      <c r="J171" s="10" t="inlineStr"/>
+      <c r="I171" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J171" s="10" t="inlineStr">
+        <is>
+          <t>CHI 1, DET 4</t>
+        </is>
+      </c>
       <c r="K171" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -9863,8 +9927,16 @@
         <f>IF(OR(F172="",G172="",AND(I172&lt;&gt;"W",I172&lt;&gt;"L")),"",IF(I172="W",IF(G172&gt;0,G172/100,1),IF(G172&lt;0,G172/100,-1)))</f>
         <v/>
       </c>
-      <c r="I172" s="11" t="inlineStr"/>
-      <c r="J172" s="10" t="inlineStr"/>
+      <c r="I172" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J172" s="10" t="inlineStr">
+        <is>
+          <t>BOS 1, STL 4</t>
+        </is>
+      </c>
       <c r="K172" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -9907,8 +9979,16 @@
         <f>IF(OR(F173="",G173="",AND(I173&lt;&gt;"W",I173&lt;&gt;"L")),"",IF(I173="W",IF(G173&gt;0,G173/100,1),IF(G173&lt;0,G173/100,-1)))</f>
         <v/>
       </c>
-      <c r="I173" s="11" t="inlineStr"/>
-      <c r="J173" s="10" t="inlineStr"/>
+      <c r="I173" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J173" s="10" t="inlineStr">
+        <is>
+          <t>WSH 4, NSH 3</t>
+        </is>
+      </c>
       <c r="K173" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -9951,8 +10031,16 @@
         <f>IF(OR(F174="",G174="",AND(I174&lt;&gt;"W",I174&lt;&gt;"L")),"",IF(I174="W",IF(G174&gt;0,G174/100,1),IF(G174&lt;0,G174/100,-1)))</f>
         <v/>
       </c>
-      <c r="I174" s="11" t="inlineStr"/>
-      <c r="J174" s="10" t="inlineStr"/>
+      <c r="I174" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J174" s="10" t="inlineStr">
+        <is>
+          <t>MTL 5, DAL 2</t>
+        </is>
+      </c>
       <c r="K174" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -9995,8 +10083,16 @@
         <f>IF(OR(F175="",G175="",AND(I175&lt;&gt;"W",I175&lt;&gt;"L")),"",IF(I175="W",IF(G175&gt;0,G175/100,1),IF(G175&lt;0,G175/100,-1)))</f>
         <v/>
       </c>
-      <c r="I175" s="11" t="inlineStr"/>
-      <c r="J175" s="10" t="inlineStr"/>
+      <c r="I175" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J175" s="10" t="inlineStr">
+        <is>
+          <t>NYI 4, MIN 3</t>
+        </is>
+      </c>
       <c r="K175" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -10039,8 +10135,16 @@
         <f>IF(OR(F176="",G176="",AND(I176&lt;&gt;"W",I176&lt;&gt;"L")),"",IF(I176="W",IF(G176&gt;0,G176/100,1),IF(G176&lt;0,G176/100,-1)))</f>
         <v/>
       </c>
-      <c r="I176" s="11" t="inlineStr"/>
-      <c r="J176" s="10" t="inlineStr"/>
+      <c r="I176" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J176" s="10" t="inlineStr">
+        <is>
+          <t>BUF 7, ANA 6</t>
+        </is>
+      </c>
       <c r="K176" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -10083,8 +10187,16 @@
         <f>IF(OR(F177="",G177="",AND(I177&lt;&gt;"W",I177&lt;&gt;"L")),"",IF(I177="W",IF(G177&gt;0,G177/100,1),IF(G177&lt;0,G177/100,-1)))</f>
         <v/>
       </c>
-      <c r="I177" s="11" t="inlineStr"/>
-      <c r="J177" s="10" t="inlineStr"/>
+      <c r="I177" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J177" s="10" t="inlineStr">
+        <is>
+          <t>OTT 5, LAK 6</t>
+        </is>
+      </c>
       <c r="K177" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -10127,8 +10239,16 @@
         <f>IF(OR(F178="",G178="",AND(I178&lt;&gt;"W",I178&lt;&gt;"L")),"",IF(I178="W",IF(G178&gt;0,G178/100,1),IF(G178&lt;0,G178/100,-1)))</f>
         <v/>
       </c>
-      <c r="I178" s="11" t="inlineStr"/>
-      <c r="J178" s="10" t="inlineStr"/>
+      <c r="I178" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J178" s="10" t="inlineStr">
+        <is>
+          <t>VAN 2, SJS 3</t>
+        </is>
+      </c>
       <c r="K178" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (4:00 PM CT)</t>
@@ -10168,7 +10288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10509,6 +10629,38 @@
       </c>
       <c r="G12" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +136 and a differential of 31.34 or less; home picks only.</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>51-19, +23.89 units</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>93-64, +12.25 units</t>
+        </is>
+      </c>
+      <c r="E13" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A13,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A13,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G13" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A13)</f>
         <v/>
       </c>
     </row>
@@ -70186,7 +70338,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-29 16:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-30 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-30 15:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$178</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$181</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -594,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -651,23 +651,23 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(F9:F33)</f>
+        <f>SUM(F9:F35)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(G9:G33,"W")/(COUNTIF(G9:G33,"W")+COUNTIF(G9:G33,"L")),"")</f>
+        <f>IFERROR(COUNTIF(G9:G35,"W")/(COUNTIF(G9:G35,"W")+COUNTIF(G9:G35,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(G9:G33,"W")&amp;"-"&amp;COUNTIF(G9:G33,"L")</f>
+        <f>COUNTIF(G9:G35,"W")&amp;"-"&amp;COUNTIF(G9:G35,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(G9:G33,"W")+COUNTIF(G9:G33,"L")</f>
+        <f>COUNTIF(G9:G35,"W")+COUNTIF(G9:G35,"L")</f>
         <v/>
       </c>
       <c r="I5" s="7">
-        <f>COUNTA(B9:B33)-COUNTIF(G9:G33,"W")-COUNTIF(G9:G33,"L")</f>
+        <f>COUNTA(B9:B35)-COUNTIF(G9:G35,"W")-COUNTIF(G9:G35,"L")</f>
         <v/>
       </c>
     </row>
@@ -1718,8 +1718,72 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="9" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>NJD @ VGK</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="n">
+        <v>-115</v>
+      </c>
+      <c r="E34" s="13" t="n">
+        <v>25.65</v>
+      </c>
+      <c r="F34" s="14">
+        <f>IF(AND(G34&lt;&gt;"W",G34&lt;&gt;"L"),"",IF(G34="W",IF(D34&gt;0,D34/100,1),IF(D34&lt;0,D34/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G34" s="11" t="inlineStr"/>
+      <c r="H34" s="10" t="inlineStr"/>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +136 and a differential of 31.34 or less; home picks only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>WPG @ FLA</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="n">
+        <v>-225</v>
+      </c>
+      <c r="E35" s="13" t="n">
+        <v>20.86</v>
+      </c>
+      <c r="F35" s="14">
+        <f>IF(AND(G35&lt;&gt;"W",G35&lt;&gt;"L"),"",IF(G35="W",IF(D35&gt;0,D35/100,1),IF(D35&lt;0,D35/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="G35" s="11" t="inlineStr"/>
+      <c r="H35" s="10" t="inlineStr"/>
+      <c r="I35" s="10" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +136 and a differential of 31.34 or less; home picks only.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:I33"/>
+  <autoFilter ref="A8:I35"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -1728,7 +1792,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F9:F33">
+  <conditionalFormatting sqref="F9:F35">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -1746,7 +1810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L178"/>
+  <dimension ref="A1:L181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1808,19 +1872,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H178)</f>
+        <f>SUM(H9:H181)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I178,"W")/(COUNTIF(I9:I178,"W")+COUNTIF(I9:I178,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I181,"W")/(COUNTIF(I9:I181,"W")+COUNTIF(I9:I181,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I178,"W")&amp;"-"&amp;COUNTIF(I9:I178,"L")</f>
+        <f>COUNTIF(I9:I181,"W")&amp;"-"&amp;COUNTIF(I9:I181,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I178,"W")+COUNTIF(I9:I178,"L")</f>
+        <f>COUNTIF(I9:I181,"W")+COUNTIF(I9:I181,"L")</f>
         <v/>
       </c>
     </row>
@@ -10260,8 +10324,140 @@
         </is>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="9" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B179" s="10" t="inlineStr">
+        <is>
+          <t>NJD @ VGK</t>
+        </is>
+      </c>
+      <c r="C179" s="13" t="n">
+        <v>47.51</v>
+      </c>
+      <c r="D179" s="13" t="n">
+        <v>73.16</v>
+      </c>
+      <c r="E179" s="13">
+        <f>IF(OR(C179="",D179=""),"",ABS(C179-D179))</f>
+        <v/>
+      </c>
+      <c r="F179" s="11" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="G179" s="12" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H179" s="14">
+        <f>IF(OR(F179="",G179="",AND(I179&lt;&gt;"W",I179&lt;&gt;"L")),"",IF(I179="W",IF(G179&gt;0,G179/100,1),IF(G179&lt;0,G179/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I179" s="11" t="inlineStr"/>
+      <c r="J179" s="10" t="inlineStr"/>
+      <c r="K179" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (3:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L179" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="9" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B180" s="10" t="inlineStr">
+        <is>
+          <t>WPG @ FLA</t>
+        </is>
+      </c>
+      <c r="C180" s="13" t="n">
+        <v>60.07</v>
+      </c>
+      <c r="D180" s="13" t="n">
+        <v>80.93000000000001</v>
+      </c>
+      <c r="E180" s="13">
+        <f>IF(OR(C180="",D180=""),"",ABS(C180-D180))</f>
+        <v/>
+      </c>
+      <c r="F180" s="11" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="G180" s="12" t="n">
+        <v>-225</v>
+      </c>
+      <c r="H180" s="14">
+        <f>IF(OR(F180="",G180="",AND(I180&lt;&gt;"W",I180&lt;&gt;"L")),"",IF(I180="W",IF(G180&gt;0,G180/100,1),IF(G180&lt;0,G180/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I180" s="11" t="inlineStr"/>
+      <c r="J180" s="10" t="inlineStr"/>
+      <c r="K180" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (3:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L180" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="9" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B181" s="10" t="inlineStr">
+        <is>
+          <t>SEA @ CGY</t>
+        </is>
+      </c>
+      <c r="C181" s="13" t="n">
+        <v>71.77</v>
+      </c>
+      <c r="D181" s="13" t="n">
+        <v>54.69</v>
+      </c>
+      <c r="E181" s="13">
+        <f>IF(OR(C181="",D181=""),"",ABS(C181-D181))</f>
+        <v/>
+      </c>
+      <c r="F181" s="11" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="G181" s="12" t="n">
+        <v>-115</v>
+      </c>
+      <c r="H181" s="14">
+        <f>IF(OR(F181="",G181="",AND(I181&lt;&gt;"W",I181&lt;&gt;"L")),"",IF(I181="W",IF(G181&gt;0,G181/100,1),IF(G181&lt;0,G181/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I181" s="11" t="inlineStr"/>
+      <c r="J181" s="10" t="inlineStr"/>
+      <c r="K181" s="10" t="inlineStr">
+        <is>
+          <t>DraftKings at pick time (3:00 PM CT)</t>
+        </is>
+      </c>
+      <c r="L181" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L178"/>
+  <autoFilter ref="A8:L181"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -10270,7 +10466,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H178">
+  <conditionalFormatting sqref="H9:H181">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -70338,7 +70534,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-30 06:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-30 15:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-31 06:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -1742,8 +1742,16 @@
         <f>IF(AND(G34&lt;&gt;"W",G34&lt;&gt;"L"),"",IF(G34="W",IF(D34&gt;0,D34/100,1),IF(D34&lt;0,D34/100,-1)))</f>
         <v/>
       </c>
-      <c r="G34" s="11" t="inlineStr"/>
-      <c r="H34" s="10" t="inlineStr"/>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>NJD 5, VGK 2</t>
+        </is>
+      </c>
       <c r="I34" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has any line up to +136 and a differential of 31.34 or less; home picks only.</t>
@@ -1774,8 +1782,16 @@
         <f>IF(AND(G35&lt;&gt;"W",G35&lt;&gt;"L"),"",IF(G35="W",IF(D35&gt;0,D35/100,1),IF(D35&lt;0,D35/100,-1)))</f>
         <v/>
       </c>
-      <c r="G35" s="11" t="inlineStr"/>
-      <c r="H35" s="10" t="inlineStr"/>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="H35" s="10" t="inlineStr">
+        <is>
+          <t>WPG 2, FLA 5</t>
+        </is>
+      </c>
       <c r="I35" s="10" t="inlineStr">
         <is>
           <t>Bet the pick when it has any line up to +136 and a differential of 31.34 or less; home picks only.</t>
@@ -1844,7 +1860,7 @@
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
-          <t>Today's rule: Bet the pick when it has any line up to +136 and a differential of 31.34 or less; home picks only.</t>
+          <t>Today's rule: Bet the pick when it has any line up to +136 and a differential of 20.86 or less; home picks only.</t>
         </is>
       </c>
     </row>
@@ -10355,8 +10371,16 @@
         <f>IF(OR(F179="",G179="",AND(I179&lt;&gt;"W",I179&lt;&gt;"L")),"",IF(I179="W",IF(G179&gt;0,G179/100,1),IF(G179&lt;0,G179/100,-1)))</f>
         <v/>
       </c>
-      <c r="I179" s="11" t="inlineStr"/>
-      <c r="J179" s="10" t="inlineStr"/>
+      <c r="I179" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J179" s="10" t="inlineStr">
+        <is>
+          <t>NJD 5, VGK 2</t>
+        </is>
+      </c>
       <c r="K179" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (3:00 PM CT)</t>
@@ -10399,8 +10423,16 @@
         <f>IF(OR(F180="",G180="",AND(I180&lt;&gt;"W",I180&lt;&gt;"L")),"",IF(I180="W",IF(G180&gt;0,G180/100,1),IF(G180&lt;0,G180/100,-1)))</f>
         <v/>
       </c>
-      <c r="I180" s="11" t="inlineStr"/>
-      <c r="J180" s="10" t="inlineStr"/>
+      <c r="I180" s="11" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="J180" s="10" t="inlineStr">
+        <is>
+          <t>WPG 2, FLA 5</t>
+        </is>
+      </c>
       <c r="K180" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (3:00 PM CT)</t>
@@ -10443,8 +10475,16 @@
         <f>IF(OR(F181="",G181="",AND(I181&lt;&gt;"W",I181&lt;&gt;"L")),"",IF(I181="W",IF(G181&gt;0,G181/100,1),IF(G181&lt;0,G181/100,-1)))</f>
         <v/>
       </c>
-      <c r="I181" s="11" t="inlineStr"/>
-      <c r="J181" s="10" t="inlineStr"/>
+      <c r="I181" s="11" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J181" s="10" t="inlineStr">
+        <is>
+          <t>SEA 2, CGY 6</t>
+        </is>
+      </c>
       <c r="K181" s="10" t="inlineStr">
         <is>
           <t>DraftKings at pick time (3:00 PM CT)</t>
@@ -10484,7 +10524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10857,6 +10897,38 @@
       </c>
       <c r="G13" s="21">
         <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Bet the pick when it has any line up to +136 and a differential of 20.86 or less; home picks only.</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>46-16, +24.04 units</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>94-66, +10.95 units</t>
+        </is>
+      </c>
+      <c r="E14" s="19">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="20">
+        <f>COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A14,'Dynamic Bet Results'!$G$9:$G$5000,"W")&amp;"-"&amp;COUNTIFS('Dynamic Bet Results'!$A$9:$A$5000,A14,'Dynamic Bet Results'!$G$9:$G$5000,"L")</f>
+        <v/>
+      </c>
+      <c r="G14" s="21">
+        <f>SUMIFS('Dynamic Bet Results'!$F$9:$F$5000,'Dynamic Bet Results'!$A$9:$A$5000,A14)</f>
         <v/>
       </c>
     </row>
@@ -70534,7 +70606,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-30 15:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-31 06:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Picks data, 2026-10-31 10:00 CT
</commit_message>
<xml_diff>
--- a/team_score_picks.xlsx
+++ b/team_score_picks.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Dynamic Bet Results'!$A$8:$I$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026-27'!$A$8:$L$191</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2025-26'!$A$8:$K$1272</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1826,7 +1826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L181"/>
+  <dimension ref="A1:L191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1888,19 +1888,19 @@
     </row>
     <row r="5">
       <c r="A5" s="4">
-        <f>SUM(H9:H181)</f>
+        <f>SUM(H9:H191)</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>IFERROR(COUNTIF(I9:I181,"W")/(COUNTIF(I9:I181,"W")+COUNTIF(I9:I181,"L")),"")</f>
+        <f>IFERROR(COUNTIF(I9:I191,"W")/(COUNTIF(I9:I191,"W")+COUNTIF(I9:I191,"L")),"")</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>COUNTIF(I9:I181,"W")&amp;"-"&amp;COUNTIF(I9:I181,"L")</f>
+        <f>COUNTIF(I9:I191,"W")&amp;"-"&amp;COUNTIF(I9:I191,"L")</f>
         <v/>
       </c>
       <c r="G5" s="7">
-        <f>COUNTIF(I9:I181,"W")+COUNTIF(I9:I181,"L")</f>
+        <f>COUNTIF(I9:I191,"W")+COUNTIF(I9:I191,"L")</f>
         <v/>
       </c>
     </row>
@@ -10496,8 +10496,428 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B182" s="10" t="inlineStr">
+        <is>
+          <t>CHI @ BOS</t>
+        </is>
+      </c>
+      <c r="C182" s="13" t="n">
+        <v>55.57</v>
+      </c>
+      <c r="D182" s="13" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="E182" s="13">
+        <f>IF(OR(C182="",D182=""),"",ABS(C182-D182))</f>
+        <v/>
+      </c>
+      <c r="F182" s="11" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="G182" s="12" t="n"/>
+      <c r="H182" s="14">
+        <f>IF(OR(F182="",G182="",AND(I182&lt;&gt;"W",I182&lt;&gt;"L")),"",IF(I182="W",IF(G182&gt;0,G182/100,1),IF(G182&lt;0,G182/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I182" s="11" t="inlineStr"/>
+      <c r="J182" s="10" t="inlineStr"/>
+      <c r="K182" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L182" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B183" s="10" t="inlineStr">
+        <is>
+          <t>STL @ DET</t>
+        </is>
+      </c>
+      <c r="C183" s="13" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="D183" s="13" t="n">
+        <v>84.43000000000001</v>
+      </c>
+      <c r="E183" s="13">
+        <f>IF(OR(C183="",D183=""),"",ABS(C183-D183))</f>
+        <v/>
+      </c>
+      <c r="F183" s="11" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="G183" s="12" t="n"/>
+      <c r="H183" s="14">
+        <f>IF(OR(F183="",G183="",AND(I183&lt;&gt;"W",I183&lt;&gt;"L")),"",IF(I183="W",IF(G183&gt;0,G183/100,1),IF(G183&lt;0,G183/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I183" s="11" t="inlineStr"/>
+      <c r="J183" s="10" t="inlineStr"/>
+      <c r="K183" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L183" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B184" s="10" t="inlineStr">
+        <is>
+          <t>TBL @ NSH</t>
+        </is>
+      </c>
+      <c r="C184" s="13" t="n">
+        <v>79.93000000000001</v>
+      </c>
+      <c r="D184" s="13" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="E184" s="13">
+        <f>IF(OR(C184="",D184=""),"",ABS(C184-D184))</f>
+        <v/>
+      </c>
+      <c r="F184" s="11" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="G184" s="12" t="n"/>
+      <c r="H184" s="14">
+        <f>IF(OR(F184="",G184="",AND(I184&lt;&gt;"W",I184&lt;&gt;"L")),"",IF(I184="W",IF(G184&gt;0,G184/100,1),IF(G184&lt;0,G184/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I184" s="11" t="inlineStr"/>
+      <c r="J184" s="10" t="inlineStr"/>
+      <c r="K184" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L184" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B185" s="10" t="inlineStr">
+        <is>
+          <t>EDM @ NYI</t>
+        </is>
+      </c>
+      <c r="C185" s="13" t="n">
+        <v>85.31</v>
+      </c>
+      <c r="D185" s="13" t="n">
+        <v>75.98999999999999</v>
+      </c>
+      <c r="E185" s="13">
+        <f>IF(OR(C185="",D185=""),"",ABS(C185-D185))</f>
+        <v/>
+      </c>
+      <c r="F185" s="11" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="G185" s="12" t="n"/>
+      <c r="H185" s="14">
+        <f>IF(OR(F185="",G185="",AND(I185&lt;&gt;"W",I185&lt;&gt;"L")),"",IF(I185="W",IF(G185&gt;0,G185/100,1),IF(G185&lt;0,G185/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I185" s="11" t="inlineStr"/>
+      <c r="J185" s="10" t="inlineStr"/>
+      <c r="K185" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L185" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B186" s="10" t="inlineStr">
+        <is>
+          <t>BUF @ LAK</t>
+        </is>
+      </c>
+      <c r="C186" s="13" t="n">
+        <v>75.79000000000001</v>
+      </c>
+      <c r="D186" s="13" t="n">
+        <v>76.97</v>
+      </c>
+      <c r="E186" s="13">
+        <f>IF(OR(C186="",D186=""),"",ABS(C186-D186))</f>
+        <v/>
+      </c>
+      <c r="F186" s="11" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="G186" s="12" t="n"/>
+      <c r="H186" s="14">
+        <f>IF(OR(F186="",G186="",AND(I186&lt;&gt;"W",I186&lt;&gt;"L")),"",IF(I186="W",IF(G186&gt;0,G186/100,1),IF(G186&lt;0,G186/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I186" s="11" t="inlineStr"/>
+      <c r="J186" s="10" t="inlineStr"/>
+      <c r="K186" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L186" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B187" s="10" t="inlineStr">
+        <is>
+          <t>OTT @ SJS</t>
+        </is>
+      </c>
+      <c r="C187" s="13" t="n">
+        <v>63.03</v>
+      </c>
+      <c r="D187" s="13" t="n">
+        <v>72.53</v>
+      </c>
+      <c r="E187" s="13">
+        <f>IF(OR(C187="",D187=""),"",ABS(C187-D187))</f>
+        <v/>
+      </c>
+      <c r="F187" s="11" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="G187" s="12" t="n"/>
+      <c r="H187" s="14">
+        <f>IF(OR(F187="",G187="",AND(I187&lt;&gt;"W",I187&lt;&gt;"L")),"",IF(I187="W",IF(G187&gt;0,G187/100,1),IF(G187&lt;0,G187/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I187" s="11" t="inlineStr"/>
+      <c r="J187" s="10" t="inlineStr"/>
+      <c r="K187" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L187" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B188" s="10" t="inlineStr">
+        <is>
+          <t>PIT @ MTL</t>
+        </is>
+      </c>
+      <c r="C188" s="13" t="n">
+        <v>63.26</v>
+      </c>
+      <c r="D188" s="13" t="n">
+        <v>79.94</v>
+      </c>
+      <c r="E188" s="13">
+        <f>IF(OR(C188="",D188=""),"",ABS(C188-D188))</f>
+        <v/>
+      </c>
+      <c r="F188" s="11" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="G188" s="12" t="n"/>
+      <c r="H188" s="14">
+        <f>IF(OR(F188="",G188="",AND(I188&lt;&gt;"W",I188&lt;&gt;"L")),"",IF(I188="W",IF(G188&gt;0,G188/100,1),IF(G188&lt;0,G188/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I188" s="11" t="inlineStr"/>
+      <c r="J188" s="10" t="inlineStr"/>
+      <c r="K188" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L188" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B189" s="10" t="inlineStr">
+        <is>
+          <t>TOR @ VAN</t>
+        </is>
+      </c>
+      <c r="C189" s="13" t="n">
+        <v>68.23</v>
+      </c>
+      <c r="D189" s="13" t="n">
+        <v>67.47</v>
+      </c>
+      <c r="E189" s="13">
+        <f>IF(OR(C189="",D189=""),"",ABS(C189-D189))</f>
+        <v/>
+      </c>
+      <c r="F189" s="11" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="G189" s="12" t="n"/>
+      <c r="H189" s="14">
+        <f>IF(OR(F189="",G189="",AND(I189&lt;&gt;"W",I189&lt;&gt;"L")),"",IF(I189="W",IF(G189&gt;0,G189/100,1),IF(G189&lt;0,G189/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I189" s="11" t="inlineStr"/>
+      <c r="J189" s="10" t="inlineStr"/>
+      <c r="K189" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L189" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B190" s="10" t="inlineStr">
+        <is>
+          <t>CBJ @ DAL</t>
+        </is>
+      </c>
+      <c r="C190" s="13" t="n">
+        <v>64.22</v>
+      </c>
+      <c r="D190" s="13" t="n">
+        <v>60.06</v>
+      </c>
+      <c r="E190" s="13">
+        <f>IF(OR(C190="",D190=""),"",ABS(C190-D190))</f>
+        <v/>
+      </c>
+      <c r="F190" s="11" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="G190" s="12" t="n"/>
+      <c r="H190" s="14">
+        <f>IF(OR(F190="",G190="",AND(I190&lt;&gt;"W",I190&lt;&gt;"L")),"",IF(I190="W",IF(G190&gt;0,G190/100,1),IF(G190&lt;0,G190/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I190" s="11" t="inlineStr"/>
+      <c r="J190" s="10" t="inlineStr"/>
+      <c r="K190" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L190" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="9" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B191" s="10" t="inlineStr">
+        <is>
+          <t>CGY @ COL</t>
+        </is>
+      </c>
+      <c r="C191" s="13" t="n">
+        <v>86.89</v>
+      </c>
+      <c r="D191" s="13" t="n">
+        <v>92.48999999999999</v>
+      </c>
+      <c r="E191" s="13">
+        <f>IF(OR(C191="",D191=""),"",ABS(C191-D191))</f>
+        <v/>
+      </c>
+      <c r="F191" s="11" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="G191" s="12" t="n"/>
+      <c r="H191" s="14">
+        <f>IF(OR(F191="",G191="",AND(I191&lt;&gt;"W",I191&lt;&gt;"L")),"",IF(I191="W",IF(G191&gt;0,G191/100,1),IF(G191&lt;0,G191/100,-1)))</f>
+        <v/>
+      </c>
+      <c r="I191" s="11" t="inlineStr"/>
+      <c r="J191" s="10" t="inlineStr"/>
+      <c r="K191" s="10" t="inlineStr">
+        <is>
+          <t>no line at pick time</t>
+        </is>
+      </c>
+      <c r="L191" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A8:L181"/>
+  <autoFilter ref="A8:L191"/>
   <conditionalFormatting sqref="A5">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
       <formula>0</formula>
@@ -10506,7 +10926,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H9:H181">
+  <conditionalFormatting sqref="H9:H191">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="2">
       <formula>0</formula>
     </cfRule>
@@ -70606,7 +71026,7 @@
       </c>
       <c r="B9" s="24" t="inlineStr">
         <is>
-          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-31 06:00 CT.</t>
+          <t>Game data: NHL public API (api-web.nhle.com). Odds: ESPN public API. Updated 2026-10-31 10:00 CT.</t>
         </is>
       </c>
     </row>

</xml_diff>